<commit_message>
Use light orange instead of yellow for duplicate lot highlight
</commit_message>
<xml_diff>
--- a/shortage_with_anode_report.xlsx
+++ b/shortage_with_anode_report.xlsx
@@ -39,8 +39,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
+        <fgColor rgb="00FFD9A0"/>
+        <bgColor rgb="00FFD9A0"/>
       </patternFill>
     </fill>
   </fills>

</xml_diff>

<commit_message>
Regenerate report with date-start 2026-08-10 and anode cutoff 2026-08-03
</commit_message>
<xml_diff>
--- a/shortage_with_anode_report.xlsx
+++ b/shortage_with_anode_report.xlsx
@@ -649,13 +649,13 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>2163114.822032</v>
+        <v>2067970.059275</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>561328</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>1601786.822032</v>
+        <v>1506642.059275</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>1074990</v>
@@ -684,13 +684,13 @@
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>901618.155774</v>
+        <v>891326.960692</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>98418</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>803200.155774</v>
+        <v>792908.960692</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>911831</v>
@@ -754,13 +754,13 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>505558.955167</v>
+        <v>479065.643072</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>166753</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>338805.955167</v>
+        <v>312312.643072</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>507119</v>
@@ -789,13 +789,13 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>312435.781968</v>
+        <v>296770.131704</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>312435.781968</v>
+        <v>296770.131704</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>98756</v>
@@ -824,13 +824,13 @@
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>363865.38971</v>
+        <v>296726.888578</v>
       </c>
       <c r="E11" s="1" t="n">
         <v>98730</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>265135.38971</v>
+        <v>197996.888578</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>98756</v>
@@ -885,25 +885,25 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>T521X226M050ATE075</t>
+          <t>T598D336M025ATE060</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>A521V116M050AS</t>
+          <t>A598D336M025AS</t>
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>40389.342806</v>
+        <v>54933.125257</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>0</v>
+        <v>16540</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>40389.342806</v>
+        <v>38393.125257</v>
       </c>
       <c r="G13" s="1" t="n">
-        <v>16157</v>
+        <v>16540</v>
       </c>
       <c r="H13" t="n">
         <v>1</v>
@@ -920,25 +920,25 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>T598D336M025ATE060</t>
+          <t>T521X226M050ATE075</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>A598D336M025AS</t>
+          <t>A521V116M050AS</t>
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>54933.125257</v>
+        <v>32880.970972</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>16540</v>
+        <v>0</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>38393.125257</v>
+        <v>32880.970972</v>
       </c>
       <c r="G14" s="1" t="n">
-        <v>16540</v>
+        <v>16157</v>
       </c>
       <c r="H14" t="n">
         <v>1</v>
@@ -14979,7 +14979,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>T521X476M035ATE030</t>
+          <t>T521X476M035ATE070</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
@@ -15011,7 +15011,7 @@
       </c>
       <c r="M198" s="2" t="inlineStr">
         <is>
-          <t>T521X476M035ATE030</t>
+          <t>T521X476M035ATE070</t>
         </is>
       </c>
       <c r="N198" s="2" t="inlineStr">
@@ -15049,7 +15049,7 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>T521X476M035ATE030</t>
+          <t>T521X476M035ATE070</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
@@ -15081,7 +15081,7 @@
       </c>
       <c r="M199" s="2" t="inlineStr">
         <is>
-          <t>T521X476M035ATE030</t>
+          <t>T521X476M035ATE070</t>
         </is>
       </c>
       <c r="N199" s="2" t="inlineStr">
@@ -15119,7 +15119,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>T521X476M035ATE030</t>
+          <t>T521X476M035ATE070</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
@@ -15151,7 +15151,7 @@
       </c>
       <c r="M200" s="2" t="inlineStr">
         <is>
-          <t>T521X476M035ATE030</t>
+          <t>T521X476M035ATE070</t>
         </is>
       </c>
       <c r="N200" s="2" t="inlineStr">
@@ -15189,7 +15189,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>T521X476M035ATE070</t>
+          <t>T521X476M035ATE030</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
@@ -15221,7 +15221,7 @@
       </c>
       <c r="M201" s="2" t="inlineStr">
         <is>
-          <t>T521X476M035ATE070</t>
+          <t>T521X476M035ATE030</t>
         </is>
       </c>
       <c r="N201" s="2" t="inlineStr">
@@ -15259,7 +15259,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>T521X476M035ATE070</t>
+          <t>T521X476M035ATE030</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
@@ -15291,7 +15291,7 @@
       </c>
       <c r="M202" s="2" t="inlineStr">
         <is>
-          <t>T521X476M035ATE070</t>
+          <t>T521X476M035ATE030</t>
         </is>
       </c>
       <c r="N202" s="2" t="inlineStr">
@@ -15329,7 +15329,7 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>T521X476M035ATE070</t>
+          <t>T521X476M035ATE030</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
@@ -15361,7 +15361,7 @@
       </c>
       <c r="M203" s="2" t="inlineStr">
         <is>
-          <t>T521X476M035ATE070</t>
+          <t>T521X476M035ATE030</t>
         </is>
       </c>
       <c r="N203" s="2" t="inlineStr">
@@ -17197,7 +17197,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
@@ -17209,7 +17209,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -17233,7 +17233,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix CoveredThroughDate to use per-row demand, not per-date aggregate
Several demand rows can share the same SUGG_START_DATE. The previous
cumulative curve summed all same-date rows into one bucket before a
date counted as covered, so a date wasn't reached until every row on
it was satisfied. That understated coverage: e.g. PlannedQty alone
already fully covers several individual 2026-09-07 rows for
T521T685M035APE0907652, so CoveredThroughDate should already read
2026-09-07 before any anode lot is even added, not stay at 2026-09-03.
Now each demand row is its own cumulative step, so a date is reported
as soon as its first row is crossed.
</commit_message>
<xml_diff>
--- a/shortage_with_anode_report.xlsx
+++ b/shortage_with_anode_report.xlsx
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1542,7 +1542,7 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1615,7 +1615,7 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1688,7 +1688,7 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1761,7 +1761,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1834,7 +1834,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -2345,7 +2345,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
@@ -2418,7 +2418,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
@@ -2491,7 +2491,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
@@ -2564,7 +2564,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
@@ -2710,7 +2710,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
@@ -2783,7 +2783,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
@@ -2856,7 +2856,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
@@ -3075,7 +3075,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
@@ -3148,7 +3148,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
@@ -3294,7 +3294,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
@@ -3367,7 +3367,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46256</v>
+        <v>46263</v>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
@@ -4096,7 +4096,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D38" s="3" t="n"/>
+      <c r="D38" s="3" t="n">
+        <v>46253</v>
+      </c>
       <c r="E38" t="inlineStr">
         <is>
           <t>2631GZ37</t>
@@ -4167,7 +4169,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D39" s="3" t="n"/>
+      <c r="D39" s="3" t="n">
+        <v>46253</v>
+      </c>
       <c r="E39" t="inlineStr">
         <is>
           <t>2631H237</t>
@@ -4238,7 +4242,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D40" s="3" t="n"/>
+      <c r="D40" s="3" t="n">
+        <v>46253</v>
+      </c>
       <c r="E40" t="inlineStr">
         <is>
           <t>2631KK47</t>
@@ -4309,7 +4315,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D41" s="3" t="n"/>
+      <c r="D41" s="3" t="n">
+        <v>46253</v>
+      </c>
       <c r="E41" t="inlineStr">
         <is>
           <t>2631HN57</t>
@@ -4380,7 +4388,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D42" s="3" t="n"/>
+      <c r="D42" s="3" t="n">
+        <v>46253</v>
+      </c>
       <c r="E42" t="inlineStr">
         <is>
           <t>2631HO27</t>
@@ -4451,7 +4461,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D43" s="3" t="n"/>
+      <c r="D43" s="3" t="n">
+        <v>46253</v>
+      </c>
       <c r="E43" t="inlineStr">
         <is>
           <t>2631KO47</t>
@@ -4522,7 +4534,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D44" s="3" t="n"/>
+      <c r="D44" s="3" t="n">
+        <v>46253</v>
+      </c>
       <c r="E44" t="inlineStr">
         <is>
           <t>2631H137</t>
@@ -4594,7 +4608,7 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46253</v>
+        <v>46258</v>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
@@ -4667,7 +4681,7 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
@@ -4740,7 +4754,7 @@
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
@@ -4813,7 +4827,7 @@
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
@@ -4959,7 +4973,7 @@
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
@@ -5032,7 +5046,7 @@
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
@@ -5105,7 +5119,7 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
@@ -5178,7 +5192,7 @@
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
@@ -5251,7 +5265,7 @@
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
@@ -5324,7 +5338,7 @@
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
@@ -5397,7 +5411,7 @@
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>46267</v>
+        <v>46272</v>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
@@ -5470,7 +5484,7 @@
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>46267</v>
+        <v>46272</v>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
@@ -5543,7 +5557,7 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>46267</v>
+        <v>46272</v>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
@@ -5616,7 +5630,7 @@
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>46267</v>
+        <v>46272</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
@@ -6199,7 +6213,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="D67" s="3" t="n"/>
+      <c r="D67" s="3" t="n">
+        <v>46256</v>
+      </c>
       <c r="E67" t="inlineStr">
         <is>
           <t>2631GM37</t>
@@ -6344,7 +6360,7 @@
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>46256</v>
+        <v>46260</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -6417,7 +6433,7 @@
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>46256</v>
+        <v>46260</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -6490,7 +6506,7 @@
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>46256</v>
+        <v>46260</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -6563,7 +6579,7 @@
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>46256</v>
+        <v>46260</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -6636,7 +6652,7 @@
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>46256</v>
+        <v>46260</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -6709,7 +6725,7 @@
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>46256</v>
+        <v>46260</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -6782,7 +6798,7 @@
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>46260</v>
+        <v>46263</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -6855,7 +6871,7 @@
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>46260</v>
+        <v>46263</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -6928,7 +6944,7 @@
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>46260</v>
+        <v>46263</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -7001,7 +7017,7 @@
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -7147,7 +7163,7 @@
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>46261</v>
+        <v>46265</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -7220,7 +7236,7 @@
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>46261</v>
+        <v>46265</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -7293,7 +7309,7 @@
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
@@ -7366,7 +7382,7 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
@@ -7439,7 +7455,7 @@
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
@@ -7512,7 +7528,7 @@
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
@@ -7585,7 +7601,7 @@
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
@@ -7658,7 +7674,7 @@
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
@@ -7731,7 +7747,7 @@
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
@@ -7804,7 +7820,7 @@
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
@@ -7877,7 +7893,7 @@
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
@@ -7950,7 +7966,7 @@
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
@@ -8023,7 +8039,7 @@
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
@@ -8096,7 +8112,7 @@
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E93" s="4" t="inlineStr">
         <is>
@@ -8169,7 +8185,7 @@
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
@@ -8242,7 +8258,7 @@
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E95" s="4" t="inlineStr">
         <is>
@@ -8315,7 +8331,7 @@
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
@@ -8388,7 +8404,7 @@
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E97" s="4" t="inlineStr">
         <is>
@@ -8461,7 +8477,7 @@
         </is>
       </c>
       <c r="D98" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
@@ -8534,7 +8550,7 @@
         </is>
       </c>
       <c r="D99" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E99" s="4" t="inlineStr">
         <is>
@@ -8607,7 +8623,7 @@
         </is>
       </c>
       <c r="D100" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
@@ -8680,7 +8696,7 @@
         </is>
       </c>
       <c r="D101" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E101" s="4" t="inlineStr">
         <is>
@@ -8753,7 +8769,7 @@
         </is>
       </c>
       <c r="D102" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
@@ -8826,7 +8842,7 @@
         </is>
       </c>
       <c r="D103" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E103" s="4" t="inlineStr">
         <is>
@@ -8899,7 +8915,7 @@
         </is>
       </c>
       <c r="D104" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
@@ -8972,7 +8988,7 @@
         </is>
       </c>
       <c r="D105" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E105" s="4" t="inlineStr">
         <is>
@@ -9045,7 +9061,7 @@
         </is>
       </c>
       <c r="D106" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
@@ -9191,7 +9207,7 @@
         </is>
       </c>
       <c r="D108" s="3" t="n">
-        <v>46258</v>
+        <v>46268</v>
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
@@ -9264,7 +9280,7 @@
         </is>
       </c>
       <c r="D109" s="3" t="n">
-        <v>46258</v>
+        <v>46268</v>
       </c>
       <c r="E109" s="4" t="inlineStr">
         <is>
@@ -9337,7 +9353,7 @@
         </is>
       </c>
       <c r="D110" s="3" t="n">
-        <v>46258</v>
+        <v>46268</v>
       </c>
       <c r="E110" s="4" t="inlineStr">
         <is>
@@ -9410,7 +9426,7 @@
         </is>
       </c>
       <c r="D111" s="3" t="n">
-        <v>46258</v>
+        <v>46268</v>
       </c>
       <c r="E111" s="4" t="inlineStr">
         <is>
@@ -9556,7 +9572,7 @@
         </is>
       </c>
       <c r="D113" s="3" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="E113" s="4" t="inlineStr">
         <is>
@@ -9629,7 +9645,7 @@
         </is>
       </c>
       <c r="D114" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E114" s="4" t="inlineStr">
         <is>
@@ -9702,7 +9718,7 @@
         </is>
       </c>
       <c r="D115" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E115" s="4" t="inlineStr">
         <is>
@@ -9775,7 +9791,7 @@
         </is>
       </c>
       <c r="D116" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
@@ -9848,7 +9864,7 @@
         </is>
       </c>
       <c r="D117" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E117" s="4" t="inlineStr">
         <is>
@@ -9921,7 +9937,7 @@
         </is>
       </c>
       <c r="D118" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
@@ -9994,7 +10010,7 @@
         </is>
       </c>
       <c r="D119" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E119" s="4" t="inlineStr">
         <is>
@@ -10067,7 +10083,7 @@
         </is>
       </c>
       <c r="D120" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
@@ -10140,7 +10156,7 @@
         </is>
       </c>
       <c r="D121" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E121" s="4" t="inlineStr">
         <is>
@@ -10213,7 +10229,7 @@
         </is>
       </c>
       <c r="D122" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
@@ -10286,7 +10302,7 @@
         </is>
       </c>
       <c r="D123" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E123" s="4" t="inlineStr">
         <is>
@@ -10359,7 +10375,7 @@
         </is>
       </c>
       <c r="D124" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E124" s="4" t="inlineStr">
         <is>
@@ -10432,7 +10448,7 @@
         </is>
       </c>
       <c r="D125" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E125" s="4" t="inlineStr">
         <is>
@@ -10505,7 +10521,7 @@
         </is>
       </c>
       <c r="D126" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E126" s="4" t="inlineStr">
         <is>
@@ -10578,7 +10594,7 @@
         </is>
       </c>
       <c r="D127" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E127" s="4" t="inlineStr">
         <is>
@@ -10651,7 +10667,7 @@
         </is>
       </c>
       <c r="D128" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E128" s="4" t="inlineStr">
         <is>
@@ -10724,7 +10740,7 @@
         </is>
       </c>
       <c r="D129" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E129" s="4" t="inlineStr">
         <is>
@@ -10797,7 +10813,7 @@
         </is>
       </c>
       <c r="D130" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E130" s="4" t="inlineStr">
         <is>
@@ -10870,7 +10886,7 @@
         </is>
       </c>
       <c r="D131" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E131" s="4" t="inlineStr">
         <is>
@@ -10943,7 +10959,7 @@
         </is>
       </c>
       <c r="D132" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E132" s="4" t="inlineStr">
         <is>
@@ -11016,7 +11032,7 @@
         </is>
       </c>
       <c r="D133" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E133" s="4" t="inlineStr">
         <is>
@@ -11089,7 +11105,7 @@
         </is>
       </c>
       <c r="D134" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E134" s="4" t="inlineStr">
         <is>
@@ -11162,7 +11178,7 @@
         </is>
       </c>
       <c r="D135" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E135" s="4" t="inlineStr">
         <is>
@@ -11235,7 +11251,7 @@
         </is>
       </c>
       <c r="D136" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E136" s="4" t="inlineStr">
         <is>
@@ -11308,7 +11324,7 @@
         </is>
       </c>
       <c r="D137" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E137" s="4" t="inlineStr">
         <is>
@@ -11381,7 +11397,7 @@
         </is>
       </c>
       <c r="D138" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E138" s="4" t="inlineStr">
         <is>
@@ -11454,7 +11470,7 @@
         </is>
       </c>
       <c r="D139" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E139" s="4" t="inlineStr">
         <is>
@@ -11527,7 +11543,7 @@
         </is>
       </c>
       <c r="D140" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E140" s="4" t="inlineStr">
         <is>
@@ -11600,7 +11616,7 @@
         </is>
       </c>
       <c r="D141" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E141" s="4" t="inlineStr">
         <is>
@@ -11673,7 +11689,7 @@
         </is>
       </c>
       <c r="D142" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E142" s="4" t="inlineStr">
         <is>
@@ -11746,7 +11762,7 @@
         </is>
       </c>
       <c r="D143" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E143" s="4" t="inlineStr">
         <is>
@@ -11819,7 +11835,7 @@
         </is>
       </c>
       <c r="D144" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E144" s="4" t="inlineStr">
         <is>
@@ -11892,7 +11908,7 @@
         </is>
       </c>
       <c r="D145" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E145" s="4" t="inlineStr">
         <is>
@@ -12621,7 +12637,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D155" s="3" t="n"/>
+      <c r="D155" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E155" s="4" t="inlineStr">
         <is>
           <t>2629UT37</t>
@@ -12692,7 +12710,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D156" s="3" t="n"/>
+      <c r="D156" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
           <t>2629LK57</t>
@@ -12763,7 +12783,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D157" s="3" t="n"/>
+      <c r="D157" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E157" s="4" t="inlineStr">
         <is>
           <t>2630OC17</t>
@@ -12834,7 +12856,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D158" s="3" t="n"/>
+      <c r="D158" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E158" s="4" t="inlineStr">
         <is>
           <t>2630SW37</t>
@@ -12905,7 +12929,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D159" s="3" t="n"/>
+      <c r="D159" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E159" s="4" t="inlineStr">
         <is>
           <t>2630SQ37</t>
@@ -12976,7 +13002,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D160" s="3" t="n"/>
+      <c r="D160" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
           <t>2630S447</t>
@@ -13047,7 +13075,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D161" s="3" t="n"/>
+      <c r="D161" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E161" s="4" t="inlineStr">
         <is>
           <t>2630QV47</t>
@@ -13118,7 +13148,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D162" s="3" t="n"/>
+      <c r="D162" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
           <t>2630S747</t>
@@ -13189,7 +13221,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D163" s="3" t="n"/>
+      <c r="D163" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E163" s="4" t="inlineStr">
         <is>
           <t>2630QY47</t>
@@ -13260,7 +13294,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D164" s="3" t="n"/>
+      <c r="D164" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
           <t>2630OB67</t>
@@ -13331,7 +13367,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D165" s="3" t="n"/>
+      <c r="D165" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E165" s="4" t="inlineStr">
         <is>
           <t>2631P427</t>
@@ -13402,7 +13440,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D166" s="3" t="n"/>
+      <c r="D166" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
           <t>2630O867</t>
@@ -13473,7 +13513,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D167" s="3" t="n"/>
+      <c r="D167" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E167" s="4" t="inlineStr">
         <is>
           <t>2630O967</t>
@@ -13544,7 +13586,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D168" s="3" t="n"/>
+      <c r="D168" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
           <t>2630OA67</t>
@@ -13615,7 +13659,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D169" s="3" t="n"/>
+      <c r="D169" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E169" s="4" t="inlineStr">
         <is>
           <t>2630OC67</t>
@@ -13686,7 +13732,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D170" s="3" t="n"/>
+      <c r="D170" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
           <t>2630OE67</t>
@@ -13757,7 +13805,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D171" s="3" t="n"/>
+      <c r="D171" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E171" s="4" t="inlineStr">
         <is>
           <t>2630OF67</t>
@@ -13828,7 +13878,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D172" s="3" t="n"/>
+      <c r="D172" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
           <t>2630OG67</t>
@@ -13899,7 +13951,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D173" s="3" t="n"/>
+      <c r="D173" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E173" s="4" t="inlineStr">
         <is>
           <t>2631ID17</t>
@@ -13970,7 +14024,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D174" s="3" t="n"/>
+      <c r="D174" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
           <t>2631IE17</t>
@@ -14041,7 +14097,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D175" s="3" t="n"/>
+      <c r="D175" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E175" s="4" t="inlineStr">
         <is>
           <t>2631IF17</t>
@@ -14112,7 +14170,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D176" s="3" t="n"/>
+      <c r="D176" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
           <t>2631IG17</t>
@@ -14183,7 +14243,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D177" s="3" t="n"/>
+      <c r="D177" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E177" s="4" t="inlineStr">
         <is>
           <t>2631IH17</t>
@@ -14254,7 +14316,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D178" s="3" t="n"/>
+      <c r="D178" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E178" s="4" t="inlineStr">
         <is>
           <t>2631II17</t>
@@ -14325,7 +14389,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D179" s="3" t="n"/>
+      <c r="D179" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
           <t>2631IJ17</t>
@@ -14396,7 +14462,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D180" s="3" t="n"/>
+      <c r="D180" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E180" s="4" t="inlineStr">
         <is>
           <t>2631IK17</t>
@@ -14467,7 +14535,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D181" s="3" t="n"/>
+      <c r="D181" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
           <t>2631OW27</t>
@@ -14538,7 +14608,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D182" s="3" t="n"/>
+      <c r="D182" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E182" s="4" t="inlineStr">
         <is>
           <t>2631OX27</t>
@@ -14609,7 +14681,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D183" s="3" t="n"/>
+      <c r="D183" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
           <t>2631OY27</t>
@@ -14680,7 +14754,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D184" s="3" t="n"/>
+      <c r="D184" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E184" s="4" t="inlineStr">
         <is>
           <t>2631OZ27</t>
@@ -14751,7 +14827,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D185" s="3" t="n"/>
+      <c r="D185" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
           <t>2631P327</t>
@@ -14822,7 +14900,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D186" s="3" t="n"/>
+      <c r="D186" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E186" s="4" t="inlineStr">
         <is>
           <t>2631P127</t>
@@ -14893,7 +14973,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D187" s="3" t="n"/>
+      <c r="D187" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
           <t>2631L237</t>
@@ -14964,7 +15046,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D188" s="3" t="n"/>
+      <c r="D188" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E188" s="4" t="inlineStr">
         <is>
           <t>2631L337</t>
@@ -15035,7 +15119,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D189" s="3" t="n"/>
+      <c r="D189" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
           <t>2631L437</t>
@@ -15106,7 +15192,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D190" s="3" t="n"/>
+      <c r="D190" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E190" s="4" t="inlineStr">
         <is>
           <t>2631OV27</t>
@@ -15177,7 +15265,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D191" s="3" t="n"/>
+      <c r="D191" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
           <t>2631P227</t>
@@ -15248,7 +15338,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D192" s="3" t="n"/>
+      <c r="D192" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E192" s="4" t="inlineStr">
         <is>
           <t>2631P627</t>
@@ -15319,7 +15411,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D193" s="3" t="n"/>
+      <c r="D193" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
           <t>2631KS37</t>
@@ -15390,7 +15484,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D194" s="3" t="n"/>
+      <c r="D194" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E194" s="4" t="inlineStr">
         <is>
           <t>2631KZ37</t>
@@ -15461,7 +15557,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D195" s="3" t="n"/>
+      <c r="D195" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
           <t>2631L137</t>
@@ -15532,7 +15630,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D196" s="3" t="n"/>
+      <c r="D196" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E196" s="4" t="inlineStr">
         <is>
           <t>2631P727</t>
@@ -15603,7 +15703,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D197" s="3" t="n"/>
+      <c r="D197" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
           <t>2631KT37</t>
@@ -15674,7 +15776,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D198" s="3" t="n"/>
+      <c r="D198" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E198" s="4" t="inlineStr">
         <is>
           <t>2631KU37</t>
@@ -15745,7 +15849,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D199" s="3" t="n"/>
+      <c r="D199" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
           <t>2631KV37</t>
@@ -15816,7 +15922,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D200" s="3" t="n"/>
+      <c r="D200" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E200" s="4" t="inlineStr">
         <is>
           <t>2631KW37</t>
@@ -15887,7 +15995,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D201" s="3" t="n"/>
+      <c r="D201" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
           <t>2631KX37</t>
@@ -15958,7 +16068,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D202" s="3" t="n"/>
+      <c r="D202" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E202" s="4" t="inlineStr">
         <is>
           <t>2631PW47</t>
@@ -16029,7 +16141,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D203" s="3" t="n"/>
+      <c r="D203" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
           <t>2631PZ47</t>
@@ -16100,7 +16214,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D204" s="3" t="n"/>
+      <c r="D204" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E204" s="4" t="inlineStr">
         <is>
           <t>2631Q147</t>
@@ -16171,7 +16287,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D205" s="3" t="n"/>
+      <c r="D205" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E205" s="4" t="inlineStr">
         <is>
           <t>2631KY37</t>
@@ -16242,7 +16360,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D206" s="3" t="n"/>
+      <c r="D206" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E206" s="4" t="inlineStr">
         <is>
           <t>2631P527</t>
@@ -16313,7 +16433,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D207" s="3" t="n"/>
+      <c r="D207" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E207" s="4" t="inlineStr">
         <is>
           <t>2631KR37</t>
@@ -16384,7 +16506,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D208" s="3" t="n"/>
+      <c r="D208" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E208" s="4" t="inlineStr">
         <is>
           <t>2631L537</t>
@@ -16455,7 +16579,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D209" s="3" t="n"/>
+      <c r="D209" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E209" s="4" t="inlineStr">
         <is>
           <t>2631L637</t>
@@ -16526,7 +16652,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D210" s="3" t="n"/>
+      <c r="D210" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E210" s="4" t="inlineStr">
         <is>
           <t>2631PX47</t>
@@ -16597,7 +16725,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D211" s="3" t="n"/>
+      <c r="D211" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E211" s="4" t="inlineStr">
         <is>
           <t>2631PY47</t>
@@ -16668,7 +16798,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D212" s="3" t="n"/>
+      <c r="D212" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E212" s="4" t="inlineStr">
         <is>
           <t>2631Q347</t>
@@ -16739,7 +16871,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D213" s="3" t="n"/>
+      <c r="D213" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E213" s="4" t="inlineStr">
         <is>
           <t>2631OJ57</t>
@@ -16810,7 +16944,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D214" s="3" t="n"/>
+      <c r="D214" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E214" s="4" t="inlineStr">
         <is>
           <t>2631OL57</t>
@@ -16881,7 +17017,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D215" s="3" t="n"/>
+      <c r="D215" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E215" s="4" t="inlineStr">
         <is>
           <t>2631ON57</t>
@@ -16952,7 +17090,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D216" s="3" t="n"/>
+      <c r="D216" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E216" s="4" t="inlineStr">
         <is>
           <t>2631FZ67</t>
@@ -17023,7 +17163,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D217" s="3" t="n"/>
+      <c r="D217" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E217" s="4" t="inlineStr">
         <is>
           <t>2631G767</t>
@@ -17094,7 +17236,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D218" s="3" t="n"/>
+      <c r="D218" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E218" s="4" t="inlineStr">
         <is>
           <t>2631Q247</t>
@@ -17165,7 +17309,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D219" s="3" t="n"/>
+      <c r="D219" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E219" s="4" t="inlineStr">
         <is>
           <t>2631Q547</t>
@@ -17236,7 +17382,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D220" s="3" t="n"/>
+      <c r="D220" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E220" s="4" t="inlineStr">
         <is>
           <t>2631OI57</t>
@@ -17307,7 +17455,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D221" s="3" t="n"/>
+      <c r="D221" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E221" s="4" t="inlineStr">
         <is>
           <t>2631OM57</t>
@@ -17378,7 +17528,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D222" s="3" t="n"/>
+      <c r="D222" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E222" s="4" t="inlineStr">
         <is>
           <t>2631OO57</t>
@@ -17449,7 +17601,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D223" s="3" t="n"/>
+      <c r="D223" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E223" s="4" t="inlineStr">
         <is>
           <t>2631G367</t>
@@ -17520,7 +17674,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D224" s="3" t="n"/>
+      <c r="D224" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E224" s="4" t="inlineStr">
         <is>
           <t>2631G467</t>
@@ -17591,7 +17747,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D225" s="3" t="n"/>
+      <c r="D225" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E225" s="4" t="inlineStr">
         <is>
           <t>2631Q447</t>
@@ -17662,7 +17820,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D226" s="3" t="n"/>
+      <c r="D226" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E226" s="4" t="inlineStr">
         <is>
           <t>2631OK57</t>
@@ -17733,7 +17893,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D227" s="3" t="n"/>
+      <c r="D227" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E227" s="4" t="inlineStr">
         <is>
           <t>2631FY67</t>
@@ -17804,7 +17966,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D228" s="3" t="n"/>
+      <c r="D228" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E228" s="4" t="inlineStr">
         <is>
           <t>2629UT37</t>
@@ -17875,7 +18039,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D229" s="3" t="n"/>
+      <c r="D229" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E229" s="4" t="inlineStr">
         <is>
           <t>2629LK57</t>
@@ -17946,7 +18112,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D230" s="3" t="n"/>
+      <c r="D230" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E230" s="4" t="inlineStr">
         <is>
           <t>2630OC17</t>
@@ -18017,7 +18185,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D231" s="3" t="n"/>
+      <c r="D231" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E231" s="4" t="inlineStr">
         <is>
           <t>2630SW37</t>
@@ -18088,7 +18258,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D232" s="3" t="n"/>
+      <c r="D232" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E232" s="4" t="inlineStr">
         <is>
           <t>2630SQ37</t>
@@ -18159,7 +18331,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D233" s="3" t="n"/>
+      <c r="D233" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E233" s="4" t="inlineStr">
         <is>
           <t>2630S447</t>
@@ -18230,7 +18404,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D234" s="3" t="n"/>
+      <c r="D234" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E234" s="4" t="inlineStr">
         <is>
           <t>2630QV47</t>
@@ -18301,7 +18477,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D235" s="3" t="n"/>
+      <c r="D235" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E235" s="4" t="inlineStr">
         <is>
           <t>2630S747</t>
@@ -18372,7 +18550,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D236" s="3" t="n"/>
+      <c r="D236" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E236" s="4" t="inlineStr">
         <is>
           <t>2630QY47</t>
@@ -18443,7 +18623,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D237" s="3" t="n"/>
+      <c r="D237" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E237" s="4" t="inlineStr">
         <is>
           <t>2630OB67</t>
@@ -18514,7 +18696,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D238" s="3" t="n"/>
+      <c r="D238" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E238" s="4" t="inlineStr">
         <is>
           <t>2631P427</t>
@@ -18585,7 +18769,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D239" s="3" t="n"/>
+      <c r="D239" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E239" s="4" t="inlineStr">
         <is>
           <t>2630O867</t>
@@ -18656,7 +18842,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D240" s="3" t="n"/>
+      <c r="D240" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E240" s="4" t="inlineStr">
         <is>
           <t>2630O967</t>
@@ -18727,7 +18915,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D241" s="3" t="n"/>
+      <c r="D241" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E241" s="4" t="inlineStr">
         <is>
           <t>2630OA67</t>
@@ -18798,7 +18988,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D242" s="3" t="n"/>
+      <c r="D242" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E242" s="4" t="inlineStr">
         <is>
           <t>2630OC67</t>
@@ -18869,7 +19061,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D243" s="3" t="n"/>
+      <c r="D243" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E243" s="4" t="inlineStr">
         <is>
           <t>2630OE67</t>
@@ -18940,7 +19134,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D244" s="3" t="n"/>
+      <c r="D244" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E244" s="4" t="inlineStr">
         <is>
           <t>2630OF67</t>
@@ -19011,7 +19207,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D245" s="3" t="n"/>
+      <c r="D245" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E245" s="4" t="inlineStr">
         <is>
           <t>2630OG67</t>
@@ -19082,7 +19280,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D246" s="3" t="n"/>
+      <c r="D246" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E246" s="4" t="inlineStr">
         <is>
           <t>2631ID17</t>
@@ -19153,7 +19353,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D247" s="3" t="n"/>
+      <c r="D247" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E247" s="4" t="inlineStr">
         <is>
           <t>2631IE17</t>
@@ -19224,7 +19426,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D248" s="3" t="n"/>
+      <c r="D248" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E248" s="4" t="inlineStr">
         <is>
           <t>2631IF17</t>
@@ -19295,7 +19499,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D249" s="3" t="n"/>
+      <c r="D249" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E249" s="4" t="inlineStr">
         <is>
           <t>2631IG17</t>
@@ -19366,7 +19572,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D250" s="3" t="n"/>
+      <c r="D250" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E250" s="4" t="inlineStr">
         <is>
           <t>2631IH17</t>
@@ -19437,7 +19645,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D251" s="3" t="n"/>
+      <c r="D251" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E251" s="4" t="inlineStr">
         <is>
           <t>2631II17</t>
@@ -19508,7 +19718,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D252" s="3" t="n"/>
+      <c r="D252" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E252" s="4" t="inlineStr">
         <is>
           <t>2631IJ17</t>
@@ -19579,7 +19791,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D253" s="3" t="n"/>
+      <c r="D253" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E253" s="4" t="inlineStr">
         <is>
           <t>2631IK17</t>
@@ -19650,7 +19864,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D254" s="3" t="n"/>
+      <c r="D254" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E254" s="4" t="inlineStr">
         <is>
           <t>2631OW27</t>
@@ -19721,7 +19937,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D255" s="3" t="n"/>
+      <c r="D255" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E255" s="4" t="inlineStr">
         <is>
           <t>2631OX27</t>
@@ -19792,7 +20010,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D256" s="3" t="n"/>
+      <c r="D256" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E256" s="4" t="inlineStr">
         <is>
           <t>2631OY27</t>
@@ -19863,7 +20083,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D257" s="3" t="n"/>
+      <c r="D257" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E257" s="4" t="inlineStr">
         <is>
           <t>2631OZ27</t>
@@ -19934,7 +20156,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D258" s="3" t="n"/>
+      <c r="D258" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E258" s="4" t="inlineStr">
         <is>
           <t>2631P327</t>
@@ -20005,7 +20229,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D259" s="3" t="n"/>
+      <c r="D259" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E259" s="4" t="inlineStr">
         <is>
           <t>2631P127</t>
@@ -20076,7 +20302,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D260" s="3" t="n"/>
+      <c r="D260" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E260" s="4" t="inlineStr">
         <is>
           <t>2631L237</t>
@@ -20147,7 +20375,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D261" s="3" t="n"/>
+      <c r="D261" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E261" s="4" t="inlineStr">
         <is>
           <t>2631L337</t>
@@ -20218,7 +20448,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D262" s="3" t="n"/>
+      <c r="D262" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E262" s="4" t="inlineStr">
         <is>
           <t>2631L437</t>
@@ -20289,7 +20521,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D263" s="3" t="n"/>
+      <c r="D263" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E263" s="4" t="inlineStr">
         <is>
           <t>2631OV27</t>
@@ -20360,7 +20594,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D264" s="3" t="n"/>
+      <c r="D264" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E264" s="4" t="inlineStr">
         <is>
           <t>2631P227</t>
@@ -20431,7 +20667,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D265" s="3" t="n"/>
+      <c r="D265" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E265" s="4" t="inlineStr">
         <is>
           <t>2631P627</t>
@@ -20502,7 +20740,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D266" s="3" t="n"/>
+      <c r="D266" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E266" s="4" t="inlineStr">
         <is>
           <t>2631KS37</t>
@@ -20573,7 +20813,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D267" s="3" t="n"/>
+      <c r="D267" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E267" s="4" t="inlineStr">
         <is>
           <t>2631KZ37</t>
@@ -20644,7 +20886,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D268" s="3" t="n"/>
+      <c r="D268" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E268" s="4" t="inlineStr">
         <is>
           <t>2631L137</t>
@@ -20715,7 +20959,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D269" s="3" t="n"/>
+      <c r="D269" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E269" s="4" t="inlineStr">
         <is>
           <t>2631P727</t>
@@ -20786,7 +21032,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D270" s="3" t="n"/>
+      <c r="D270" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E270" s="4" t="inlineStr">
         <is>
           <t>2631KT37</t>
@@ -20857,7 +21105,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D271" s="3" t="n"/>
+      <c r="D271" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E271" s="4" t="inlineStr">
         <is>
           <t>2631KU37</t>
@@ -20928,7 +21178,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D272" s="3" t="n"/>
+      <c r="D272" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E272" s="4" t="inlineStr">
         <is>
           <t>2631KV37</t>
@@ -20999,7 +21251,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D273" s="3" t="n"/>
+      <c r="D273" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E273" s="4" t="inlineStr">
         <is>
           <t>2631KW37</t>
@@ -21070,7 +21324,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D274" s="3" t="n"/>
+      <c r="D274" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E274" s="4" t="inlineStr">
         <is>
           <t>2631KX37</t>
@@ -21141,7 +21397,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D275" s="3" t="n"/>
+      <c r="D275" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E275" s="4" t="inlineStr">
         <is>
           <t>2631PW47</t>
@@ -21212,7 +21470,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D276" s="3" t="n"/>
+      <c r="D276" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E276" s="4" t="inlineStr">
         <is>
           <t>2631PZ47</t>
@@ -21283,7 +21543,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D277" s="3" t="n"/>
+      <c r="D277" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E277" s="4" t="inlineStr">
         <is>
           <t>2631Q147</t>
@@ -21354,7 +21616,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D278" s="3" t="n"/>
+      <c r="D278" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E278" s="4" t="inlineStr">
         <is>
           <t>2631KY37</t>
@@ -21425,7 +21689,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D279" s="3" t="n"/>
+      <c r="D279" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E279" s="4" t="inlineStr">
         <is>
           <t>2631P527</t>
@@ -21496,7 +21762,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D280" s="3" t="n"/>
+      <c r="D280" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E280" s="4" t="inlineStr">
         <is>
           <t>2631KR37</t>
@@ -21567,7 +21835,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D281" s="3" t="n"/>
+      <c r="D281" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E281" s="4" t="inlineStr">
         <is>
           <t>2631L537</t>
@@ -21638,7 +21908,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D282" s="3" t="n"/>
+      <c r="D282" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E282" s="4" t="inlineStr">
         <is>
           <t>2631L637</t>
@@ -21709,7 +21981,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D283" s="3" t="n"/>
+      <c r="D283" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E283" s="4" t="inlineStr">
         <is>
           <t>2631PX47</t>
@@ -21780,7 +22054,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D284" s="3" t="n"/>
+      <c r="D284" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E284" s="4" t="inlineStr">
         <is>
           <t>2631PY47</t>
@@ -21851,7 +22127,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D285" s="3" t="n"/>
+      <c r="D285" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E285" s="4" t="inlineStr">
         <is>
           <t>2631Q347</t>
@@ -21922,7 +22200,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D286" s="3" t="n"/>
+      <c r="D286" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E286" s="4" t="inlineStr">
         <is>
           <t>2631OJ57</t>
@@ -21993,7 +22273,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D287" s="3" t="n"/>
+      <c r="D287" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E287" s="4" t="inlineStr">
         <is>
           <t>2631OL57</t>
@@ -22064,7 +22346,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D288" s="3" t="n"/>
+      <c r="D288" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E288" s="4" t="inlineStr">
         <is>
           <t>2631ON57</t>
@@ -22135,7 +22419,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D289" s="3" t="n"/>
+      <c r="D289" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E289" s="4" t="inlineStr">
         <is>
           <t>2631FZ67</t>
@@ -22206,7 +22492,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D290" s="3" t="n"/>
+      <c r="D290" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E290" s="4" t="inlineStr">
         <is>
           <t>2631G767</t>
@@ -22277,7 +22565,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D291" s="3" t="n"/>
+      <c r="D291" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E291" s="4" t="inlineStr">
         <is>
           <t>2631Q247</t>
@@ -22348,7 +22638,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D292" s="3" t="n"/>
+      <c r="D292" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E292" s="4" t="inlineStr">
         <is>
           <t>2631Q547</t>
@@ -22419,7 +22711,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D293" s="3" t="n"/>
+      <c r="D293" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E293" s="4" t="inlineStr">
         <is>
           <t>2631OI57</t>
@@ -22490,7 +22784,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D294" s="3" t="n"/>
+      <c r="D294" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E294" s="4" t="inlineStr">
         <is>
           <t>2631OM57</t>
@@ -22561,7 +22857,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D295" s="3" t="n"/>
+      <c r="D295" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E295" s="4" t="inlineStr">
         <is>
           <t>2631OO57</t>
@@ -22632,7 +22930,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D296" s="3" t="n"/>
+      <c r="D296" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E296" s="4" t="inlineStr">
         <is>
           <t>2631G367</t>
@@ -22703,7 +23003,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D297" s="3" t="n"/>
+      <c r="D297" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E297" s="4" t="inlineStr">
         <is>
           <t>2631G467</t>
@@ -22774,7 +23076,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D298" s="3" t="n"/>
+      <c r="D298" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E298" s="4" t="inlineStr">
         <is>
           <t>2631Q447</t>
@@ -22845,7 +23149,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D299" s="3" t="n"/>
+      <c r="D299" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E299" s="4" t="inlineStr">
         <is>
           <t>2631OK57</t>
@@ -22916,7 +23222,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D300" s="3" t="n"/>
+      <c r="D300" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E300" s="4" t="inlineStr">
         <is>
           <t>2631FY67</t>
@@ -23200,7 +23508,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D304" s="3" t="n"/>
+      <c r="D304" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E304" t="inlineStr">
         <is>
           <t>2628FU10</t>
@@ -23271,7 +23581,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D305" s="3" t="n"/>
+      <c r="D305" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E305" t="inlineStr">
         <is>
           <t>2630FY20</t>
@@ -23342,7 +23654,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D306" s="3" t="n"/>
+      <c r="D306" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E306" t="inlineStr">
         <is>
           <t>2630FY30</t>
@@ -23414,7 +23728,7 @@
         </is>
       </c>
       <c r="D307" s="3" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="E307" s="4" t="inlineStr">
         <is>
@@ -23487,7 +23801,7 @@
         </is>
       </c>
       <c r="D308" s="3" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="E308" s="4" t="inlineStr">
         <is>
@@ -23560,7 +23874,7 @@
         </is>
       </c>
       <c r="D309" s="3" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="E309" s="4" t="inlineStr">
         <is>
@@ -23633,7 +23947,7 @@
         </is>
       </c>
       <c r="D310" s="3" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="E310" s="4" t="inlineStr">
         <is>
@@ -23706,7 +24020,7 @@
         </is>
       </c>
       <c r="D311" s="3" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="E311" s="4" t="inlineStr">
         <is>
@@ -23779,7 +24093,7 @@
         </is>
       </c>
       <c r="D312" s="3" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="E312" s="4" t="inlineStr">
         <is>
@@ -23852,7 +24166,7 @@
         </is>
       </c>
       <c r="D313" s="3" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="E313" s="4" t="inlineStr">
         <is>
@@ -23925,7 +24239,7 @@
         </is>
       </c>
       <c r="D314" s="3" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="E314" s="4" t="inlineStr">
         <is>
@@ -23998,7 +24312,7 @@
         </is>
       </c>
       <c r="D315" s="3" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="E315" s="4" t="inlineStr">
         <is>
@@ -24071,7 +24385,7 @@
         </is>
       </c>
       <c r="D316" s="3" t="n">
-        <v>46262</v>
+        <v>46272</v>
       </c>
       <c r="E316" s="4" t="inlineStr">
         <is>
@@ -24144,7 +24458,7 @@
         </is>
       </c>
       <c r="D317" s="3" t="n">
-        <v>46262</v>
+        <v>46272</v>
       </c>
       <c r="E317" s="4" t="inlineStr">
         <is>
@@ -24217,7 +24531,7 @@
         </is>
       </c>
       <c r="D318" s="3" t="n">
-        <v>46262</v>
+        <v>46272</v>
       </c>
       <c r="E318" s="4" t="inlineStr">
         <is>
@@ -26109,7 +26423,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D344" s="3" t="n"/>
+      <c r="D344" s="3" t="n">
+        <v>46262</v>
+      </c>
       <c r="E344" s="4" t="inlineStr">
         <is>
           <t>2630L757</t>
@@ -26181,7 +26497,7 @@
         </is>
       </c>
       <c r="D345" s="3" t="n">
-        <v>46256</v>
+        <v>46261</v>
       </c>
       <c r="E345" s="4" t="inlineStr">
         <is>
@@ -26254,7 +26570,7 @@
         </is>
       </c>
       <c r="D346" s="3" t="n">
-        <v>46256</v>
+        <v>46261</v>
       </c>
       <c r="E346" s="4" t="inlineStr">
         <is>
@@ -26327,7 +26643,7 @@
         </is>
       </c>
       <c r="D347" s="3" t="n">
-        <v>46256</v>
+        <v>46261</v>
       </c>
       <c r="E347" s="4" t="inlineStr">
         <is>
@@ -26400,7 +26716,7 @@
         </is>
       </c>
       <c r="D348" s="3" t="n">
-        <v>46256</v>
+        <v>46261</v>
       </c>
       <c r="E348" s="4" t="inlineStr">
         <is>
@@ -26473,7 +26789,7 @@
         </is>
       </c>
       <c r="D349" s="3" t="n">
-        <v>46256</v>
+        <v>46261</v>
       </c>
       <c r="E349" s="4" t="inlineStr">
         <is>
@@ -26546,7 +26862,7 @@
         </is>
       </c>
       <c r="D350" s="3" t="n">
-        <v>46256</v>
+        <v>46261</v>
       </c>
       <c r="E350" s="4" t="inlineStr">
         <is>
@@ -26619,7 +26935,7 @@
         </is>
       </c>
       <c r="D351" s="3" t="n">
-        <v>46256</v>
+        <v>46261</v>
       </c>
       <c r="E351" s="4" t="inlineStr">
         <is>
@@ -26765,7 +27081,7 @@
         </is>
       </c>
       <c r="D353" s="3" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="E353" s="4" t="inlineStr">
         <is>
@@ -26838,7 +27154,7 @@
         </is>
       </c>
       <c r="D354" s="3" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="E354" s="4" t="inlineStr">
         <is>
@@ -26911,7 +27227,7 @@
         </is>
       </c>
       <c r="D355" s="3" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="E355" s="4" t="inlineStr">
         <is>
@@ -28515,7 +28831,7 @@
         </is>
       </c>
       <c r="D377" s="3" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -28588,7 +28904,7 @@
         </is>
       </c>
       <c r="D378" s="3" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="E378" t="inlineStr">
         <is>
@@ -28734,7 +29050,7 @@
         </is>
       </c>
       <c r="D380" s="3" t="n">
-        <v>46258</v>
+        <v>46268</v>
       </c>
       <c r="E380" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Base CoveredThroughDate on the part's full order backlog, not just the near-term demand window
RequiredQty/ShortageQty (and which parts qualify as short) still use
only the demand rows inside date_start..date_end, but CoveredThroughDate
was also capped at date_end, so it could never advance past the window
even when supply clearly reached further out. get_demand now also
collects each part's full set of demand rows (AE > threshold, any date)
and CoveredThroughDate is computed against that instead.

Verified against the reported example: for T521T685M035APE0907652, the
10th lot (2609GZ57) now correctly reads 2026-09-13, matching the manual
calculation (338331 + 42029 lots + 166753 planned = 547113, which lands
just past the first 2026-09-13 demand row at cumulative 546193.79).
</commit_message>
<xml_diff>
--- a/shortage_with_anode_report.xlsx
+++ b/shortage_with_anode_report.xlsx
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46272</v>
+        <v>46278</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -2126,7 +2126,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46272</v>
+        <v>46278</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2199,7 +2199,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46272</v>
+        <v>46278</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2272,7 +2272,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46272</v>
+        <v>46278</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -3513,7 +3513,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46272</v>
+        <v>46278</v>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
@@ -3586,7 +3586,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46272</v>
+        <v>46278</v>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
@@ -3659,7 +3659,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46272</v>
+        <v>46278</v>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
@@ -3732,7 +3732,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46272</v>
+        <v>46278</v>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
@@ -3805,7 +3805,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46272</v>
+        <v>46278</v>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
@@ -3878,7 +3878,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46272</v>
+        <v>46278</v>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
@@ -4024,7 +4024,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46263</v>
+        <v>46277</v>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
@@ -5703,7 +5703,7 @@
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>46272</v>
+        <v>46276</v>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
@@ -5776,7 +5776,7 @@
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>46272</v>
+        <v>46277</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
@@ -5849,7 +5849,7 @@
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>46272</v>
+        <v>46277</v>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
@@ -5922,7 +5922,7 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>46272</v>
+        <v>46277</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
@@ -5995,7 +5995,7 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>46272</v>
+        <v>46277</v>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>46272</v>
+        <v>46279</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
@@ -6141,7 +6141,7 @@
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>46272</v>
+        <v>46281</v>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
@@ -12054,7 +12054,7 @@
         </is>
       </c>
       <c r="D147" s="3" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="E147" s="4" t="inlineStr">
         <is>
@@ -12127,7 +12127,7 @@
         </is>
       </c>
       <c r="D148" s="3" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
@@ -12200,7 +12200,7 @@
         </is>
       </c>
       <c r="D149" s="3" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="E149" s="4" t="inlineStr">
         <is>
@@ -12273,7 +12273,7 @@
         </is>
       </c>
       <c r="D150" s="3" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="E150" s="4" t="inlineStr">
         <is>
@@ -12346,7 +12346,7 @@
         </is>
       </c>
       <c r="D151" s="3" t="n">
-        <v>46275</v>
+        <v>46282</v>
       </c>
       <c r="E151" s="4" t="inlineStr">
         <is>
@@ -12419,7 +12419,7 @@
         </is>
       </c>
       <c r="D152" s="3" t="n">
-        <v>46275</v>
+        <v>46282</v>
       </c>
       <c r="E152" s="4" t="inlineStr">
         <is>
@@ -12492,7 +12492,7 @@
         </is>
       </c>
       <c r="D153" s="3" t="n">
-        <v>46275</v>
+        <v>46282</v>
       </c>
       <c r="E153" s="4" t="inlineStr">
         <is>
@@ -12565,7 +12565,7 @@
         </is>
       </c>
       <c r="D154" s="3" t="n">
-        <v>46275</v>
+        <v>46282</v>
       </c>
       <c r="E154" s="4" t="inlineStr">
         <is>
@@ -24604,7 +24604,7 @@
         </is>
       </c>
       <c r="D319" s="3" t="n">
-        <v>46271</v>
+        <v>46279</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -24677,7 +24677,7 @@
         </is>
       </c>
       <c r="D320" s="3" t="n">
-        <v>46271</v>
+        <v>46279</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -24745,7 +24745,7 @@
         </is>
       </c>
       <c r="D321" s="3" t="n">
-        <v>46271</v>
+        <v>46279</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -24818,7 +24818,7 @@
         </is>
       </c>
       <c r="D322" s="3" t="n">
-        <v>46271</v>
+        <v>46279</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -24891,7 +24891,7 @@
         </is>
       </c>
       <c r="D323" s="3" t="n">
-        <v>46271</v>
+        <v>46279</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -24964,7 +24964,7 @@
         </is>
       </c>
       <c r="D324" s="3" t="n">
-        <v>46271</v>
+        <v>46279</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -25037,7 +25037,7 @@
         </is>
       </c>
       <c r="D325" s="3" t="n">
-        <v>46271</v>
+        <v>46279</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -25110,7 +25110,7 @@
         </is>
       </c>
       <c r="D326" s="3" t="n">
-        <v>46271</v>
+        <v>46287</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -25183,7 +25183,7 @@
         </is>
       </c>
       <c r="D327" s="3" t="n">
-        <v>46271</v>
+        <v>46287</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -25256,7 +25256,7 @@
         </is>
       </c>
       <c r="D328" s="3" t="n">
-        <v>46271</v>
+        <v>46287</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -25329,7 +25329,7 @@
         </is>
       </c>
       <c r="D329" s="3" t="n">
-        <v>46271</v>
+        <v>46287</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -25402,7 +25402,7 @@
         </is>
       </c>
       <c r="D330" s="3" t="n">
-        <v>46271</v>
+        <v>46287</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -25475,7 +25475,7 @@
         </is>
       </c>
       <c r="D331" s="3" t="n">
-        <v>46271</v>
+        <v>46287</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -25548,7 +25548,7 @@
         </is>
       </c>
       <c r="D332" s="3" t="n">
-        <v>46271</v>
+        <v>46287</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -25621,7 +25621,7 @@
         </is>
       </c>
       <c r="D333" s="3" t="n">
-        <v>46271</v>
+        <v>46287</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -25694,7 +25694,7 @@
         </is>
       </c>
       <c r="D334" s="3" t="n">
-        <v>46271</v>
+        <v>46287</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -25767,7 +25767,7 @@
         </is>
       </c>
       <c r="D335" s="3" t="n">
-        <v>46271</v>
+        <v>46287</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -25840,7 +25840,7 @@
         </is>
       </c>
       <c r="D336" s="3" t="n">
-        <v>46271</v>
+        <v>46287</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -25913,7 +25913,7 @@
         </is>
       </c>
       <c r="D337" s="3" t="n">
-        <v>46271</v>
+        <v>46287</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -25986,7 +25986,7 @@
         </is>
       </c>
       <c r="D338" s="3" t="n">
-        <v>46271</v>
+        <v>46287</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -26059,7 +26059,7 @@
         </is>
       </c>
       <c r="D339" s="3" t="n">
-        <v>46271</v>
+        <v>46287</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -26132,7 +26132,7 @@
         </is>
       </c>
       <c r="D340" s="3" t="n">
-        <v>46271</v>
+        <v>46287</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -26205,7 +26205,7 @@
         </is>
       </c>
       <c r="D341" s="3" t="n">
-        <v>46271</v>
+        <v>46287</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -26278,7 +26278,7 @@
         </is>
       </c>
       <c r="D342" s="3" t="n">
-        <v>46271</v>
+        <v>46287</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -26351,7 +26351,7 @@
         </is>
       </c>
       <c r="D343" s="3" t="n">
-        <v>46271</v>
+        <v>46287</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -28466,7 +28466,7 @@
         </is>
       </c>
       <c r="D372" s="3" t="n">
-        <v>46274</v>
+        <v>46282</v>
       </c>
       <c r="E372" t="inlineStr">
         <is>
@@ -28539,7 +28539,7 @@
         </is>
       </c>
       <c r="D373" s="3" t="n">
-        <v>46274</v>
+        <v>46282</v>
       </c>
       <c r="E373" t="inlineStr">
         <is>
@@ -28612,7 +28612,7 @@
         </is>
       </c>
       <c r="D374" s="3" t="n">
-        <v>46274</v>
+        <v>46282</v>
       </c>
       <c r="E374" t="inlineStr">
         <is>
@@ -28685,7 +28685,7 @@
         </is>
       </c>
       <c r="D375" s="3" t="n">
-        <v>46274</v>
+        <v>46282</v>
       </c>
       <c r="E375" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Switch CoveredThroughDate to require the full day's demand satisfied
Previous per-row rule marked a date as covered as soon as cumulative
supply crossed any single row on it, even if other rows sharing that
date were still unmet. Confirmed against a new example
(T521B156M025ATE100): supply of 710,102 crosses 9 of 8/26's 10 rows
but not all of it (needs 729,170), so CoveredThroughDate should stay
at 2026-08-22 until the 9th lot pushes supply to 760,862 - only then
does 2026-08-26 count as covered. That directly conflicts with the
per-row rule, which reported 2026-08-26 one lot early.

build_cumulative_demand now aggregates all rows sharing a
SUGG_START_DATE into one step again, so a date only counts once every
row on it is fully satisfied. This regresses the two earlier verified
examples (T521T685M035APE0907652: lot 1 to 2026-09-03, lot 10 to
2026-09-11) per explicit instruction to use the full-day rule
consistently rather than mixing rules across examples.
</commit_message>
<xml_diff>
--- a/shortage_with_anode_report.xlsx
+++ b/shortage_with_anode_report.xlsx
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46272</v>
+        <v>46268</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1542,7 +1542,7 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46272</v>
+        <v>46268</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1615,7 +1615,7 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46272</v>
+        <v>46268</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1688,7 +1688,7 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46272</v>
+        <v>46268</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1761,7 +1761,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46272</v>
+        <v>46268</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1834,7 +1834,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46272</v>
+        <v>46268</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46272</v>
+        <v>46268</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46278</v>
+        <v>46276</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -2126,7 +2126,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46278</v>
+        <v>46276</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2199,7 +2199,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46278</v>
+        <v>46276</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2272,7 +2272,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46278</v>
+        <v>46276</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2345,7 +2345,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46262</v>
+        <v>46255</v>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
@@ -2418,7 +2418,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46262</v>
+        <v>46255</v>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
@@ -2491,7 +2491,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46262</v>
+        <v>46255</v>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
@@ -2564,7 +2564,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46262</v>
+        <v>46255</v>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
@@ -2710,7 +2710,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46268</v>
+        <v>46262</v>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
@@ -2783,7 +2783,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46268</v>
+        <v>46262</v>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
@@ -2856,7 +2856,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46268</v>
+        <v>46262</v>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46268</v>
+        <v>46262</v>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46268</v>
+        <v>46262</v>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
@@ -3075,7 +3075,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46268</v>
+        <v>46262</v>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
@@ -3148,7 +3148,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46268</v>
+        <v>46262</v>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
@@ -3294,7 +3294,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46272</v>
+        <v>46268</v>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
@@ -3367,7 +3367,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46272</v>
+        <v>46268</v>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
@@ -3513,7 +3513,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46278</v>
+        <v>46272</v>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
@@ -3586,7 +3586,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46278</v>
+        <v>46272</v>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
@@ -3659,7 +3659,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46278</v>
+        <v>46272</v>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
@@ -3732,7 +3732,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46278</v>
+        <v>46272</v>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
@@ -3805,7 +3805,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46278</v>
+        <v>46272</v>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
@@ -3878,7 +3878,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46278</v>
+        <v>46272</v>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46263</v>
+        <v>46256</v>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
@@ -4096,9 +4096,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D38" s="3" t="n">
-        <v>46253</v>
-      </c>
+      <c r="D38" s="3" t="n"/>
       <c r="E38" t="inlineStr">
         <is>
           <t>2631GZ37</t>
@@ -4169,9 +4167,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D39" s="3" t="n">
-        <v>46253</v>
-      </c>
+      <c r="D39" s="3" t="n"/>
       <c r="E39" t="inlineStr">
         <is>
           <t>2631H237</t>
@@ -4242,9 +4238,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D40" s="3" t="n">
-        <v>46253</v>
-      </c>
+      <c r="D40" s="3" t="n"/>
       <c r="E40" t="inlineStr">
         <is>
           <t>2631KK47</t>
@@ -4315,9 +4309,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D41" s="3" t="n">
-        <v>46253</v>
-      </c>
+      <c r="D41" s="3" t="n"/>
       <c r="E41" t="inlineStr">
         <is>
           <t>2631HN57</t>
@@ -4388,9 +4380,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D42" s="3" t="n">
-        <v>46253</v>
-      </c>
+      <c r="D42" s="3" t="n"/>
       <c r="E42" t="inlineStr">
         <is>
           <t>2631HO27</t>
@@ -4461,9 +4451,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D43" s="3" t="n">
-        <v>46253</v>
-      </c>
+      <c r="D43" s="3" t="n"/>
       <c r="E43" t="inlineStr">
         <is>
           <t>2631KO47</t>
@@ -4534,9 +4522,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D44" s="3" t="n">
-        <v>46253</v>
-      </c>
+      <c r="D44" s="3" t="n"/>
       <c r="E44" t="inlineStr">
         <is>
           <t>2631H137</t>
@@ -4608,7 +4594,7 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46258</v>
+        <v>46253</v>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
@@ -4681,7 +4667,7 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46265</v>
+        <v>46262</v>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
@@ -4754,7 +4740,7 @@
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46265</v>
+        <v>46262</v>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
@@ -4827,7 +4813,7 @@
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46265</v>
+        <v>46262</v>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
@@ -4973,7 +4959,7 @@
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>46267</v>
+        <v>46265</v>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
@@ -5046,7 +5032,7 @@
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>46267</v>
+        <v>46265</v>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
@@ -5119,7 +5105,7 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>46267</v>
+        <v>46265</v>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
@@ -5192,7 +5178,7 @@
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>46267</v>
+        <v>46265</v>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
@@ -5265,7 +5251,7 @@
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>46267</v>
+        <v>46265</v>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
@@ -5338,7 +5324,7 @@
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>46267</v>
+        <v>46265</v>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
@@ -5411,7 +5397,7 @@
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>46272</v>
+        <v>46267</v>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
@@ -5484,7 +5470,7 @@
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>46272</v>
+        <v>46267</v>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
@@ -5557,7 +5543,7 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>46272</v>
+        <v>46267</v>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
@@ -5630,7 +5616,7 @@
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>46272</v>
+        <v>46267</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
@@ -5776,7 +5762,7 @@
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
@@ -5849,7 +5835,7 @@
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
@@ -5922,7 +5908,7 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
@@ -5995,7 +5981,7 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
@@ -6141,7 +6127,7 @@
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>46281</v>
+        <v>46279</v>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
@@ -6213,9 +6199,7 @@
           <t>P</t>
         </is>
       </c>
-      <c r="D67" s="3" t="n">
-        <v>46256</v>
-      </c>
+      <c r="D67" s="3" t="n"/>
       <c r="E67" t="inlineStr">
         <is>
           <t>2631GM37</t>
@@ -6360,7 +6344,7 @@
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>46260</v>
+        <v>46256</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -6433,7 +6417,7 @@
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>46260</v>
+        <v>46256</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -6506,7 +6490,7 @@
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>46260</v>
+        <v>46256</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -6579,7 +6563,7 @@
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>46260</v>
+        <v>46256</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -6652,7 +6636,7 @@
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>46260</v>
+        <v>46256</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -6725,7 +6709,7 @@
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>46260</v>
+        <v>46256</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -6798,7 +6782,7 @@
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>46263</v>
+        <v>46260</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -6871,7 +6855,7 @@
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>46263</v>
+        <v>46260</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -6944,7 +6928,7 @@
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>46263</v>
+        <v>46260</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -7017,7 +7001,7 @@
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -7163,7 +7147,7 @@
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>46265</v>
+        <v>46261</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -7236,7 +7220,7 @@
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>46265</v>
+        <v>46261</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -7309,7 +7293,7 @@
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
@@ -7382,7 +7366,7 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
@@ -7455,7 +7439,7 @@
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
@@ -7528,7 +7512,7 @@
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
@@ -7601,7 +7585,7 @@
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
@@ -7674,7 +7658,7 @@
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
@@ -7747,7 +7731,7 @@
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
@@ -7820,7 +7804,7 @@
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
@@ -7893,7 +7877,7 @@
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
@@ -7966,7 +7950,7 @@
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
@@ -8039,7 +8023,7 @@
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
@@ -8112,7 +8096,7 @@
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E93" s="4" t="inlineStr">
         <is>
@@ -8185,7 +8169,7 @@
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
@@ -8258,7 +8242,7 @@
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E95" s="4" t="inlineStr">
         <is>
@@ -8331,7 +8315,7 @@
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
@@ -8404,7 +8388,7 @@
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E97" s="4" t="inlineStr">
         <is>
@@ -8477,7 +8461,7 @@
         </is>
       </c>
       <c r="D98" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
@@ -8550,7 +8534,7 @@
         </is>
       </c>
       <c r="D99" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E99" s="4" t="inlineStr">
         <is>
@@ -8623,7 +8607,7 @@
         </is>
       </c>
       <c r="D100" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
@@ -8696,7 +8680,7 @@
         </is>
       </c>
       <c r="D101" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E101" s="4" t="inlineStr">
         <is>
@@ -8769,7 +8753,7 @@
         </is>
       </c>
       <c r="D102" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
@@ -8842,7 +8826,7 @@
         </is>
       </c>
       <c r="D103" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E103" s="4" t="inlineStr">
         <is>
@@ -8915,7 +8899,7 @@
         </is>
       </c>
       <c r="D104" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
@@ -8988,7 +8972,7 @@
         </is>
       </c>
       <c r="D105" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E105" s="4" t="inlineStr">
         <is>
@@ -9061,7 +9045,7 @@
         </is>
       </c>
       <c r="D106" s="3" t="n">
-        <v>46258</v>
+        <v>46257</v>
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
@@ -9207,7 +9191,7 @@
         </is>
       </c>
       <c r="D108" s="3" t="n">
-        <v>46268</v>
+        <v>46258</v>
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
@@ -9280,7 +9264,7 @@
         </is>
       </c>
       <c r="D109" s="3" t="n">
-        <v>46268</v>
+        <v>46258</v>
       </c>
       <c r="E109" s="4" t="inlineStr">
         <is>
@@ -9353,7 +9337,7 @@
         </is>
       </c>
       <c r="D110" s="3" t="n">
-        <v>46268</v>
+        <v>46258</v>
       </c>
       <c r="E110" s="4" t="inlineStr">
         <is>
@@ -9426,7 +9410,7 @@
         </is>
       </c>
       <c r="D111" s="3" t="n">
-        <v>46268</v>
+        <v>46258</v>
       </c>
       <c r="E111" s="4" t="inlineStr">
         <is>
@@ -9572,7 +9556,7 @@
         </is>
       </c>
       <c r="D113" s="3" t="n">
-        <v>46272</v>
+        <v>46268</v>
       </c>
       <c r="E113" s="4" t="inlineStr">
         <is>
@@ -9645,7 +9629,7 @@
         </is>
       </c>
       <c r="D114" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E114" s="4" t="inlineStr">
         <is>
@@ -9718,7 +9702,7 @@
         </is>
       </c>
       <c r="D115" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E115" s="4" t="inlineStr">
         <is>
@@ -9791,7 +9775,7 @@
         </is>
       </c>
       <c r="D116" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
@@ -9864,7 +9848,7 @@
         </is>
       </c>
       <c r="D117" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E117" s="4" t="inlineStr">
         <is>
@@ -9937,7 +9921,7 @@
         </is>
       </c>
       <c r="D118" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
@@ -10010,7 +9994,7 @@
         </is>
       </c>
       <c r="D119" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E119" s="4" t="inlineStr">
         <is>
@@ -10083,7 +10067,7 @@
         </is>
       </c>
       <c r="D120" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
@@ -10156,7 +10140,7 @@
         </is>
       </c>
       <c r="D121" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E121" s="4" t="inlineStr">
         <is>
@@ -10229,7 +10213,7 @@
         </is>
       </c>
       <c r="D122" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
@@ -10302,7 +10286,7 @@
         </is>
       </c>
       <c r="D123" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E123" s="4" t="inlineStr">
         <is>
@@ -10375,7 +10359,7 @@
         </is>
       </c>
       <c r="D124" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E124" s="4" t="inlineStr">
         <is>
@@ -10448,7 +10432,7 @@
         </is>
       </c>
       <c r="D125" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E125" s="4" t="inlineStr">
         <is>
@@ -10521,7 +10505,7 @@
         </is>
       </c>
       <c r="D126" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E126" s="4" t="inlineStr">
         <is>
@@ -10594,7 +10578,7 @@
         </is>
       </c>
       <c r="D127" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E127" s="4" t="inlineStr">
         <is>
@@ -10667,7 +10651,7 @@
         </is>
       </c>
       <c r="D128" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E128" s="4" t="inlineStr">
         <is>
@@ -10740,7 +10724,7 @@
         </is>
       </c>
       <c r="D129" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E129" s="4" t="inlineStr">
         <is>
@@ -10813,7 +10797,7 @@
         </is>
       </c>
       <c r="D130" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E130" s="4" t="inlineStr">
         <is>
@@ -10886,7 +10870,7 @@
         </is>
       </c>
       <c r="D131" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E131" s="4" t="inlineStr">
         <is>
@@ -10959,7 +10943,7 @@
         </is>
       </c>
       <c r="D132" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E132" s="4" t="inlineStr">
         <is>
@@ -11032,7 +11016,7 @@
         </is>
       </c>
       <c r="D133" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E133" s="4" t="inlineStr">
         <is>
@@ -11105,7 +11089,7 @@
         </is>
       </c>
       <c r="D134" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E134" s="4" t="inlineStr">
         <is>
@@ -11178,7 +11162,7 @@
         </is>
       </c>
       <c r="D135" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E135" s="4" t="inlineStr">
         <is>
@@ -11251,7 +11235,7 @@
         </is>
       </c>
       <c r="D136" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E136" s="4" t="inlineStr">
         <is>
@@ -11324,7 +11308,7 @@
         </is>
       </c>
       <c r="D137" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E137" s="4" t="inlineStr">
         <is>
@@ -11397,7 +11381,7 @@
         </is>
       </c>
       <c r="D138" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E138" s="4" t="inlineStr">
         <is>
@@ -11470,7 +11454,7 @@
         </is>
       </c>
       <c r="D139" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E139" s="4" t="inlineStr">
         <is>
@@ -11543,7 +11527,7 @@
         </is>
       </c>
       <c r="D140" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E140" s="4" t="inlineStr">
         <is>
@@ -11616,7 +11600,7 @@
         </is>
       </c>
       <c r="D141" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E141" s="4" t="inlineStr">
         <is>
@@ -11689,7 +11673,7 @@
         </is>
       </c>
       <c r="D142" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E142" s="4" t="inlineStr">
         <is>
@@ -11762,7 +11746,7 @@
         </is>
       </c>
       <c r="D143" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E143" s="4" t="inlineStr">
         <is>
@@ -11835,7 +11819,7 @@
         </is>
       </c>
       <c r="D144" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E144" s="4" t="inlineStr">
         <is>
@@ -11908,7 +11892,7 @@
         </is>
       </c>
       <c r="D145" s="3" t="n">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="E145" s="4" t="inlineStr">
         <is>
@@ -12054,7 +12038,7 @@
         </is>
       </c>
       <c r="D147" s="3" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="E147" s="4" t="inlineStr">
         <is>
@@ -12127,7 +12111,7 @@
         </is>
       </c>
       <c r="D148" s="3" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
@@ -12200,7 +12184,7 @@
         </is>
       </c>
       <c r="D149" s="3" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="E149" s="4" t="inlineStr">
         <is>
@@ -12346,7 +12330,7 @@
         </is>
       </c>
       <c r="D151" s="3" t="n">
-        <v>46282</v>
+        <v>46276</v>
       </c>
       <c r="E151" s="4" t="inlineStr">
         <is>
@@ -12419,7 +12403,7 @@
         </is>
       </c>
       <c r="D152" s="3" t="n">
-        <v>46282</v>
+        <v>46276</v>
       </c>
       <c r="E152" s="4" t="inlineStr">
         <is>
@@ -12492,7 +12476,7 @@
         </is>
       </c>
       <c r="D153" s="3" t="n">
-        <v>46282</v>
+        <v>46276</v>
       </c>
       <c r="E153" s="4" t="inlineStr">
         <is>
@@ -12565,7 +12549,7 @@
         </is>
       </c>
       <c r="D154" s="3" t="n">
-        <v>46282</v>
+        <v>46276</v>
       </c>
       <c r="E154" s="4" t="inlineStr">
         <is>
@@ -12637,9 +12621,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D155" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D155" s="3" t="n"/>
       <c r="E155" s="4" t="inlineStr">
         <is>
           <t>2629UT37</t>
@@ -12710,9 +12692,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D156" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D156" s="3" t="n"/>
       <c r="E156" s="4" t="inlineStr">
         <is>
           <t>2629LK57</t>
@@ -12783,9 +12763,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D157" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D157" s="3" t="n"/>
       <c r="E157" s="4" t="inlineStr">
         <is>
           <t>2630OC17</t>
@@ -12856,9 +12834,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D158" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D158" s="3" t="n"/>
       <c r="E158" s="4" t="inlineStr">
         <is>
           <t>2630SW37</t>
@@ -12929,9 +12905,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D159" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D159" s="3" t="n"/>
       <c r="E159" s="4" t="inlineStr">
         <is>
           <t>2630SQ37</t>
@@ -13002,9 +12976,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D160" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D160" s="3" t="n"/>
       <c r="E160" s="4" t="inlineStr">
         <is>
           <t>2630S447</t>
@@ -13075,9 +13047,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D161" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D161" s="3" t="n"/>
       <c r="E161" s="4" t="inlineStr">
         <is>
           <t>2630QV47</t>
@@ -13148,9 +13118,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D162" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D162" s="3" t="n"/>
       <c r="E162" s="4" t="inlineStr">
         <is>
           <t>2630S747</t>
@@ -13221,9 +13189,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D163" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D163" s="3" t="n"/>
       <c r="E163" s="4" t="inlineStr">
         <is>
           <t>2630QY47</t>
@@ -13294,9 +13260,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D164" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D164" s="3" t="n"/>
       <c r="E164" s="4" t="inlineStr">
         <is>
           <t>2630OB67</t>
@@ -13367,9 +13331,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D165" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D165" s="3" t="n"/>
       <c r="E165" s="4" t="inlineStr">
         <is>
           <t>2631P427</t>
@@ -13440,9 +13402,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D166" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D166" s="3" t="n"/>
       <c r="E166" s="4" t="inlineStr">
         <is>
           <t>2630O867</t>
@@ -13513,9 +13473,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D167" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D167" s="3" t="n"/>
       <c r="E167" s="4" t="inlineStr">
         <is>
           <t>2630O967</t>
@@ -13586,9 +13544,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D168" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D168" s="3" t="n"/>
       <c r="E168" s="4" t="inlineStr">
         <is>
           <t>2630OA67</t>
@@ -13659,9 +13615,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D169" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D169" s="3" t="n"/>
       <c r="E169" s="4" t="inlineStr">
         <is>
           <t>2630OC67</t>
@@ -13732,9 +13686,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D170" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D170" s="3" t="n"/>
       <c r="E170" s="4" t="inlineStr">
         <is>
           <t>2630OE67</t>
@@ -13805,9 +13757,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D171" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D171" s="3" t="n"/>
       <c r="E171" s="4" t="inlineStr">
         <is>
           <t>2630OF67</t>
@@ -13878,9 +13828,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D172" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D172" s="3" t="n"/>
       <c r="E172" s="4" t="inlineStr">
         <is>
           <t>2630OG67</t>
@@ -13951,9 +13899,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D173" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D173" s="3" t="n"/>
       <c r="E173" s="4" t="inlineStr">
         <is>
           <t>2631ID17</t>
@@ -14024,9 +13970,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D174" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D174" s="3" t="n"/>
       <c r="E174" s="4" t="inlineStr">
         <is>
           <t>2631IE17</t>
@@ -14097,9 +14041,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D175" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D175" s="3" t="n"/>
       <c r="E175" s="4" t="inlineStr">
         <is>
           <t>2631IF17</t>
@@ -14170,9 +14112,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D176" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D176" s="3" t="n"/>
       <c r="E176" s="4" t="inlineStr">
         <is>
           <t>2631IG17</t>
@@ -14243,9 +14183,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D177" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D177" s="3" t="n"/>
       <c r="E177" s="4" t="inlineStr">
         <is>
           <t>2631IH17</t>
@@ -14316,9 +14254,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D178" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D178" s="3" t="n"/>
       <c r="E178" s="4" t="inlineStr">
         <is>
           <t>2631II17</t>
@@ -14389,9 +14325,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D179" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D179" s="3" t="n"/>
       <c r="E179" s="4" t="inlineStr">
         <is>
           <t>2631IJ17</t>
@@ -14462,9 +14396,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D180" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D180" s="3" t="n"/>
       <c r="E180" s="4" t="inlineStr">
         <is>
           <t>2631IK17</t>
@@ -14535,9 +14467,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D181" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D181" s="3" t="n"/>
       <c r="E181" s="4" t="inlineStr">
         <is>
           <t>2631OW27</t>
@@ -14608,9 +14538,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D182" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D182" s="3" t="n"/>
       <c r="E182" s="4" t="inlineStr">
         <is>
           <t>2631OX27</t>
@@ -14681,9 +14609,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D183" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D183" s="3" t="n"/>
       <c r="E183" s="4" t="inlineStr">
         <is>
           <t>2631OY27</t>
@@ -14754,9 +14680,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D184" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D184" s="3" t="n"/>
       <c r="E184" s="4" t="inlineStr">
         <is>
           <t>2631OZ27</t>
@@ -14827,9 +14751,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D185" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D185" s="3" t="n"/>
       <c r="E185" s="4" t="inlineStr">
         <is>
           <t>2631P327</t>
@@ -14900,9 +14822,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D186" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D186" s="3" t="n"/>
       <c r="E186" s="4" t="inlineStr">
         <is>
           <t>2631P127</t>
@@ -14973,9 +14893,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D187" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D187" s="3" t="n"/>
       <c r="E187" s="4" t="inlineStr">
         <is>
           <t>2631L237</t>
@@ -15046,9 +14964,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D188" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D188" s="3" t="n"/>
       <c r="E188" s="4" t="inlineStr">
         <is>
           <t>2631L337</t>
@@ -15119,9 +15035,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D189" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D189" s="3" t="n"/>
       <c r="E189" s="4" t="inlineStr">
         <is>
           <t>2631L437</t>
@@ -15192,9 +15106,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D190" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D190" s="3" t="n"/>
       <c r="E190" s="4" t="inlineStr">
         <is>
           <t>2631OV27</t>
@@ -15265,9 +15177,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D191" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D191" s="3" t="n"/>
       <c r="E191" s="4" t="inlineStr">
         <is>
           <t>2631P227</t>
@@ -15338,9 +15248,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D192" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D192" s="3" t="n"/>
       <c r="E192" s="4" t="inlineStr">
         <is>
           <t>2631P627</t>
@@ -15411,9 +15319,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D193" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D193" s="3" t="n"/>
       <c r="E193" s="4" t="inlineStr">
         <is>
           <t>2631KS37</t>
@@ -15484,9 +15390,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D194" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D194" s="3" t="n"/>
       <c r="E194" s="4" t="inlineStr">
         <is>
           <t>2631KZ37</t>
@@ -15557,9 +15461,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D195" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D195" s="3" t="n"/>
       <c r="E195" s="4" t="inlineStr">
         <is>
           <t>2631L137</t>
@@ -15630,9 +15532,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D196" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D196" s="3" t="n"/>
       <c r="E196" s="4" t="inlineStr">
         <is>
           <t>2631P727</t>
@@ -15703,9 +15603,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D197" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D197" s="3" t="n"/>
       <c r="E197" s="4" t="inlineStr">
         <is>
           <t>2631KT37</t>
@@ -15776,9 +15674,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D198" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D198" s="3" t="n"/>
       <c r="E198" s="4" t="inlineStr">
         <is>
           <t>2631KU37</t>
@@ -15849,9 +15745,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D199" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D199" s="3" t="n"/>
       <c r="E199" s="4" t="inlineStr">
         <is>
           <t>2631KV37</t>
@@ -15922,9 +15816,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D200" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D200" s="3" t="n"/>
       <c r="E200" s="4" t="inlineStr">
         <is>
           <t>2631KW37</t>
@@ -15995,9 +15887,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D201" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D201" s="3" t="n"/>
       <c r="E201" s="4" t="inlineStr">
         <is>
           <t>2631KX37</t>
@@ -16068,9 +15958,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D202" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D202" s="3" t="n"/>
       <c r="E202" s="4" t="inlineStr">
         <is>
           <t>2631PW47</t>
@@ -16141,9 +16029,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D203" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D203" s="3" t="n"/>
       <c r="E203" s="4" t="inlineStr">
         <is>
           <t>2631PZ47</t>
@@ -16214,9 +16100,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D204" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D204" s="3" t="n"/>
       <c r="E204" s="4" t="inlineStr">
         <is>
           <t>2631Q147</t>
@@ -16287,9 +16171,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D205" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D205" s="3" t="n"/>
       <c r="E205" s="4" t="inlineStr">
         <is>
           <t>2631KY37</t>
@@ -16360,9 +16242,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D206" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D206" s="3" t="n"/>
       <c r="E206" s="4" t="inlineStr">
         <is>
           <t>2631P527</t>
@@ -16433,9 +16313,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D207" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D207" s="3" t="n"/>
       <c r="E207" s="4" t="inlineStr">
         <is>
           <t>2631KR37</t>
@@ -16506,9 +16384,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D208" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D208" s="3" t="n"/>
       <c r="E208" s="4" t="inlineStr">
         <is>
           <t>2631L537</t>
@@ -16579,9 +16455,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D209" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D209" s="3" t="n"/>
       <c r="E209" s="4" t="inlineStr">
         <is>
           <t>2631L637</t>
@@ -16652,9 +16526,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D210" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D210" s="3" t="n"/>
       <c r="E210" s="4" t="inlineStr">
         <is>
           <t>2631PX47</t>
@@ -16725,9 +16597,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D211" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D211" s="3" t="n"/>
       <c r="E211" s="4" t="inlineStr">
         <is>
           <t>2631PY47</t>
@@ -16798,9 +16668,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D212" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D212" s="3" t="n"/>
       <c r="E212" s="4" t="inlineStr">
         <is>
           <t>2631Q347</t>
@@ -16871,9 +16739,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D213" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D213" s="3" t="n"/>
       <c r="E213" s="4" t="inlineStr">
         <is>
           <t>2631OJ57</t>
@@ -16944,9 +16810,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D214" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D214" s="3" t="n"/>
       <c r="E214" s="4" t="inlineStr">
         <is>
           <t>2631OL57</t>
@@ -17017,9 +16881,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D215" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D215" s="3" t="n"/>
       <c r="E215" s="4" t="inlineStr">
         <is>
           <t>2631ON57</t>
@@ -17090,9 +16952,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D216" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D216" s="3" t="n"/>
       <c r="E216" s="4" t="inlineStr">
         <is>
           <t>2631FZ67</t>
@@ -17163,9 +17023,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D217" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D217" s="3" t="n"/>
       <c r="E217" s="4" t="inlineStr">
         <is>
           <t>2631G767</t>
@@ -17236,9 +17094,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D218" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D218" s="3" t="n"/>
       <c r="E218" s="4" t="inlineStr">
         <is>
           <t>2631Q247</t>
@@ -17309,9 +17165,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D219" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D219" s="3" t="n"/>
       <c r="E219" s="4" t="inlineStr">
         <is>
           <t>2631Q547</t>
@@ -17382,9 +17236,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D220" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D220" s="3" t="n"/>
       <c r="E220" s="4" t="inlineStr">
         <is>
           <t>2631OI57</t>
@@ -17455,9 +17307,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D221" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D221" s="3" t="n"/>
       <c r="E221" s="4" t="inlineStr">
         <is>
           <t>2631OM57</t>
@@ -17528,9 +17378,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D222" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D222" s="3" t="n"/>
       <c r="E222" s="4" t="inlineStr">
         <is>
           <t>2631OO57</t>
@@ -17601,9 +17449,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D223" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D223" s="3" t="n"/>
       <c r="E223" s="4" t="inlineStr">
         <is>
           <t>2631G367</t>
@@ -17674,9 +17520,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D224" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D224" s="3" t="n"/>
       <c r="E224" s="4" t="inlineStr">
         <is>
           <t>2631G467</t>
@@ -17747,9 +17591,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D225" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D225" s="3" t="n"/>
       <c r="E225" s="4" t="inlineStr">
         <is>
           <t>2631Q447</t>
@@ -17820,9 +17662,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D226" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D226" s="3" t="n"/>
       <c r="E226" s="4" t="inlineStr">
         <is>
           <t>2631OK57</t>
@@ -17893,9 +17733,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D227" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D227" s="3" t="n"/>
       <c r="E227" s="4" t="inlineStr">
         <is>
           <t>2631FY67</t>
@@ -17966,9 +17804,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D228" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D228" s="3" t="n"/>
       <c r="E228" s="4" t="inlineStr">
         <is>
           <t>2629UT37</t>
@@ -18039,9 +17875,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D229" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D229" s="3" t="n"/>
       <c r="E229" s="4" t="inlineStr">
         <is>
           <t>2629LK57</t>
@@ -18112,9 +17946,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D230" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D230" s="3" t="n"/>
       <c r="E230" s="4" t="inlineStr">
         <is>
           <t>2630OC17</t>
@@ -18185,9 +18017,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D231" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D231" s="3" t="n"/>
       <c r="E231" s="4" t="inlineStr">
         <is>
           <t>2630SW37</t>
@@ -18258,9 +18088,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D232" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D232" s="3" t="n"/>
       <c r="E232" s="4" t="inlineStr">
         <is>
           <t>2630SQ37</t>
@@ -18331,9 +18159,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D233" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D233" s="3" t="n"/>
       <c r="E233" s="4" t="inlineStr">
         <is>
           <t>2630S447</t>
@@ -18404,9 +18230,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D234" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D234" s="3" t="n"/>
       <c r="E234" s="4" t="inlineStr">
         <is>
           <t>2630QV47</t>
@@ -18477,9 +18301,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D235" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D235" s="3" t="n"/>
       <c r="E235" s="4" t="inlineStr">
         <is>
           <t>2630S747</t>
@@ -18550,9 +18372,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D236" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D236" s="3" t="n"/>
       <c r="E236" s="4" t="inlineStr">
         <is>
           <t>2630QY47</t>
@@ -18623,9 +18443,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D237" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D237" s="3" t="n"/>
       <c r="E237" s="4" t="inlineStr">
         <is>
           <t>2630OB67</t>
@@ -18696,9 +18514,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D238" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D238" s="3" t="n"/>
       <c r="E238" s="4" t="inlineStr">
         <is>
           <t>2631P427</t>
@@ -18769,9 +18585,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D239" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D239" s="3" t="n"/>
       <c r="E239" s="4" t="inlineStr">
         <is>
           <t>2630O867</t>
@@ -18842,9 +18656,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D240" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D240" s="3" t="n"/>
       <c r="E240" s="4" t="inlineStr">
         <is>
           <t>2630O967</t>
@@ -18915,9 +18727,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D241" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D241" s="3" t="n"/>
       <c r="E241" s="4" t="inlineStr">
         <is>
           <t>2630OA67</t>
@@ -18988,9 +18798,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D242" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D242" s="3" t="n"/>
       <c r="E242" s="4" t="inlineStr">
         <is>
           <t>2630OC67</t>
@@ -19061,9 +18869,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D243" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D243" s="3" t="n"/>
       <c r="E243" s="4" t="inlineStr">
         <is>
           <t>2630OE67</t>
@@ -19134,9 +18940,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D244" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D244" s="3" t="n"/>
       <c r="E244" s="4" t="inlineStr">
         <is>
           <t>2630OF67</t>
@@ -19207,9 +19011,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D245" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D245" s="3" t="n"/>
       <c r="E245" s="4" t="inlineStr">
         <is>
           <t>2630OG67</t>
@@ -19280,9 +19082,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D246" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D246" s="3" t="n"/>
       <c r="E246" s="4" t="inlineStr">
         <is>
           <t>2631ID17</t>
@@ -19353,9 +19153,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D247" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D247" s="3" t="n"/>
       <c r="E247" s="4" t="inlineStr">
         <is>
           <t>2631IE17</t>
@@ -19426,9 +19224,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D248" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D248" s="3" t="n"/>
       <c r="E248" s="4" t="inlineStr">
         <is>
           <t>2631IF17</t>
@@ -19499,9 +19295,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D249" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D249" s="3" t="n"/>
       <c r="E249" s="4" t="inlineStr">
         <is>
           <t>2631IG17</t>
@@ -19572,9 +19366,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D250" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D250" s="3" t="n"/>
       <c r="E250" s="4" t="inlineStr">
         <is>
           <t>2631IH17</t>
@@ -19645,9 +19437,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D251" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D251" s="3" t="n"/>
       <c r="E251" s="4" t="inlineStr">
         <is>
           <t>2631II17</t>
@@ -19718,9 +19508,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D252" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D252" s="3" t="n"/>
       <c r="E252" s="4" t="inlineStr">
         <is>
           <t>2631IJ17</t>
@@ -19791,9 +19579,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D253" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D253" s="3" t="n"/>
       <c r="E253" s="4" t="inlineStr">
         <is>
           <t>2631IK17</t>
@@ -19864,9 +19650,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D254" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D254" s="3" t="n"/>
       <c r="E254" s="4" t="inlineStr">
         <is>
           <t>2631OW27</t>
@@ -19937,9 +19721,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D255" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D255" s="3" t="n"/>
       <c r="E255" s="4" t="inlineStr">
         <is>
           <t>2631OX27</t>
@@ -20010,9 +19792,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D256" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D256" s="3" t="n"/>
       <c r="E256" s="4" t="inlineStr">
         <is>
           <t>2631OY27</t>
@@ -20083,9 +19863,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D257" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D257" s="3" t="n"/>
       <c r="E257" s="4" t="inlineStr">
         <is>
           <t>2631OZ27</t>
@@ -20156,9 +19934,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D258" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D258" s="3" t="n"/>
       <c r="E258" s="4" t="inlineStr">
         <is>
           <t>2631P327</t>
@@ -20229,9 +20005,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D259" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D259" s="3" t="n"/>
       <c r="E259" s="4" t="inlineStr">
         <is>
           <t>2631P127</t>
@@ -20302,9 +20076,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D260" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D260" s="3" t="n"/>
       <c r="E260" s="4" t="inlineStr">
         <is>
           <t>2631L237</t>
@@ -20375,9 +20147,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D261" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D261" s="3" t="n"/>
       <c r="E261" s="4" t="inlineStr">
         <is>
           <t>2631L337</t>
@@ -20448,9 +20218,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D262" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D262" s="3" t="n"/>
       <c r="E262" s="4" t="inlineStr">
         <is>
           <t>2631L437</t>
@@ -20521,9 +20289,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D263" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D263" s="3" t="n"/>
       <c r="E263" s="4" t="inlineStr">
         <is>
           <t>2631OV27</t>
@@ -20594,9 +20360,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D264" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D264" s="3" t="n"/>
       <c r="E264" s="4" t="inlineStr">
         <is>
           <t>2631P227</t>
@@ -20667,9 +20431,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D265" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D265" s="3" t="n"/>
       <c r="E265" s="4" t="inlineStr">
         <is>
           <t>2631P627</t>
@@ -20740,9 +20502,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D266" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D266" s="3" t="n"/>
       <c r="E266" s="4" t="inlineStr">
         <is>
           <t>2631KS37</t>
@@ -20813,9 +20573,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D267" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D267" s="3" t="n"/>
       <c r="E267" s="4" t="inlineStr">
         <is>
           <t>2631KZ37</t>
@@ -20886,9 +20644,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D268" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D268" s="3" t="n"/>
       <c r="E268" s="4" t="inlineStr">
         <is>
           <t>2631L137</t>
@@ -20959,9 +20715,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D269" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D269" s="3" t="n"/>
       <c r="E269" s="4" t="inlineStr">
         <is>
           <t>2631P727</t>
@@ -21032,9 +20786,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D270" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D270" s="3" t="n"/>
       <c r="E270" s="4" t="inlineStr">
         <is>
           <t>2631KT37</t>
@@ -21105,9 +20857,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D271" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D271" s="3" t="n"/>
       <c r="E271" s="4" t="inlineStr">
         <is>
           <t>2631KU37</t>
@@ -21178,9 +20928,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D272" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D272" s="3" t="n"/>
       <c r="E272" s="4" t="inlineStr">
         <is>
           <t>2631KV37</t>
@@ -21251,9 +20999,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D273" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D273" s="3" t="n"/>
       <c r="E273" s="4" t="inlineStr">
         <is>
           <t>2631KW37</t>
@@ -21324,9 +21070,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D274" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D274" s="3" t="n"/>
       <c r="E274" s="4" t="inlineStr">
         <is>
           <t>2631KX37</t>
@@ -21397,9 +21141,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D275" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D275" s="3" t="n"/>
       <c r="E275" s="4" t="inlineStr">
         <is>
           <t>2631PW47</t>
@@ -21470,9 +21212,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D276" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D276" s="3" t="n"/>
       <c r="E276" s="4" t="inlineStr">
         <is>
           <t>2631PZ47</t>
@@ -21543,9 +21283,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D277" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D277" s="3" t="n"/>
       <c r="E277" s="4" t="inlineStr">
         <is>
           <t>2631Q147</t>
@@ -21616,9 +21354,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D278" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D278" s="3" t="n"/>
       <c r="E278" s="4" t="inlineStr">
         <is>
           <t>2631KY37</t>
@@ -21689,9 +21425,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D279" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D279" s="3" t="n"/>
       <c r="E279" s="4" t="inlineStr">
         <is>
           <t>2631P527</t>
@@ -21762,9 +21496,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D280" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D280" s="3" t="n"/>
       <c r="E280" s="4" t="inlineStr">
         <is>
           <t>2631KR37</t>
@@ -21835,9 +21567,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D281" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D281" s="3" t="n"/>
       <c r="E281" s="4" t="inlineStr">
         <is>
           <t>2631L537</t>
@@ -21908,9 +21638,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D282" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D282" s="3" t="n"/>
       <c r="E282" s="4" t="inlineStr">
         <is>
           <t>2631L637</t>
@@ -21981,9 +21709,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D283" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D283" s="3" t="n"/>
       <c r="E283" s="4" t="inlineStr">
         <is>
           <t>2631PX47</t>
@@ -22054,9 +21780,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D284" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D284" s="3" t="n"/>
       <c r="E284" s="4" t="inlineStr">
         <is>
           <t>2631PY47</t>
@@ -22127,9 +21851,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D285" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D285" s="3" t="n"/>
       <c r="E285" s="4" t="inlineStr">
         <is>
           <t>2631Q347</t>
@@ -22200,9 +21922,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D286" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D286" s="3" t="n"/>
       <c r="E286" s="4" t="inlineStr">
         <is>
           <t>2631OJ57</t>
@@ -22273,9 +21993,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D287" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D287" s="3" t="n"/>
       <c r="E287" s="4" t="inlineStr">
         <is>
           <t>2631OL57</t>
@@ -22346,9 +22064,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D288" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D288" s="3" t="n"/>
       <c r="E288" s="4" t="inlineStr">
         <is>
           <t>2631ON57</t>
@@ -22419,9 +22135,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D289" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D289" s="3" t="n"/>
       <c r="E289" s="4" t="inlineStr">
         <is>
           <t>2631FZ67</t>
@@ -22492,9 +22206,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D290" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D290" s="3" t="n"/>
       <c r="E290" s="4" t="inlineStr">
         <is>
           <t>2631G767</t>
@@ -22565,9 +22277,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D291" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D291" s="3" t="n"/>
       <c r="E291" s="4" t="inlineStr">
         <is>
           <t>2631Q247</t>
@@ -22638,9 +22348,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D292" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D292" s="3" t="n"/>
       <c r="E292" s="4" t="inlineStr">
         <is>
           <t>2631Q547</t>
@@ -22711,9 +22419,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D293" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D293" s="3" t="n"/>
       <c r="E293" s="4" t="inlineStr">
         <is>
           <t>2631OI57</t>
@@ -22784,9 +22490,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D294" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D294" s="3" t="n"/>
       <c r="E294" s="4" t="inlineStr">
         <is>
           <t>2631OM57</t>
@@ -22857,9 +22561,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D295" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D295" s="3" t="n"/>
       <c r="E295" s="4" t="inlineStr">
         <is>
           <t>2631OO57</t>
@@ -22930,9 +22632,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D296" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D296" s="3" t="n"/>
       <c r="E296" s="4" t="inlineStr">
         <is>
           <t>2631G367</t>
@@ -23003,9 +22703,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D297" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D297" s="3" t="n"/>
       <c r="E297" s="4" t="inlineStr">
         <is>
           <t>2631G467</t>
@@ -23076,9 +22774,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D298" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D298" s="3" t="n"/>
       <c r="E298" s="4" t="inlineStr">
         <is>
           <t>2631Q447</t>
@@ -23149,9 +22845,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D299" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D299" s="3" t="n"/>
       <c r="E299" s="4" t="inlineStr">
         <is>
           <t>2631OK57</t>
@@ -23222,9 +22916,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D300" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D300" s="3" t="n"/>
       <c r="E300" s="4" t="inlineStr">
         <is>
           <t>2631FY67</t>
@@ -23508,9 +23200,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D304" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D304" s="3" t="n"/>
       <c r="E304" t="inlineStr">
         <is>
           <t>2628FU10</t>
@@ -23581,9 +23271,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D305" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D305" s="3" t="n"/>
       <c r="E305" t="inlineStr">
         <is>
           <t>2630FY20</t>
@@ -23654,9 +23342,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D306" s="3" t="n">
-        <v>46258</v>
-      </c>
+      <c r="D306" s="3" t="n"/>
       <c r="E306" t="inlineStr">
         <is>
           <t>2630FY30</t>
@@ -23728,7 +23414,7 @@
         </is>
       </c>
       <c r="D307" s="3" t="n">
-        <v>46262</v>
+        <v>46255</v>
       </c>
       <c r="E307" s="4" t="inlineStr">
         <is>
@@ -23801,7 +23487,7 @@
         </is>
       </c>
       <c r="D308" s="3" t="n">
-        <v>46262</v>
+        <v>46255</v>
       </c>
       <c r="E308" s="4" t="inlineStr">
         <is>
@@ -23874,7 +23560,7 @@
         </is>
       </c>
       <c r="D309" s="3" t="n">
-        <v>46262</v>
+        <v>46255</v>
       </c>
       <c r="E309" s="4" t="inlineStr">
         <is>
@@ -23947,7 +23633,7 @@
         </is>
       </c>
       <c r="D310" s="3" t="n">
-        <v>46262</v>
+        <v>46255</v>
       </c>
       <c r="E310" s="4" t="inlineStr">
         <is>
@@ -24020,7 +23706,7 @@
         </is>
       </c>
       <c r="D311" s="3" t="n">
-        <v>46262</v>
+        <v>46255</v>
       </c>
       <c r="E311" s="4" t="inlineStr">
         <is>
@@ -24093,7 +23779,7 @@
         </is>
       </c>
       <c r="D312" s="3" t="n">
-        <v>46262</v>
+        <v>46255</v>
       </c>
       <c r="E312" s="4" t="inlineStr">
         <is>
@@ -24166,7 +23852,7 @@
         </is>
       </c>
       <c r="D313" s="3" t="n">
-        <v>46262</v>
+        <v>46260</v>
       </c>
       <c r="E313" s="4" t="inlineStr">
         <is>
@@ -24239,7 +23925,7 @@
         </is>
       </c>
       <c r="D314" s="3" t="n">
-        <v>46262</v>
+        <v>46260</v>
       </c>
       <c r="E314" s="4" t="inlineStr">
         <is>
@@ -24312,7 +23998,7 @@
         </is>
       </c>
       <c r="D315" s="3" t="n">
-        <v>46262</v>
+        <v>46260</v>
       </c>
       <c r="E315" s="4" t="inlineStr">
         <is>
@@ -24385,7 +24071,7 @@
         </is>
       </c>
       <c r="D316" s="3" t="n">
-        <v>46272</v>
+        <v>46262</v>
       </c>
       <c r="E316" s="4" t="inlineStr">
         <is>
@@ -24458,7 +24144,7 @@
         </is>
       </c>
       <c r="D317" s="3" t="n">
-        <v>46272</v>
+        <v>46262</v>
       </c>
       <c r="E317" s="4" t="inlineStr">
         <is>
@@ -24531,7 +24217,7 @@
         </is>
       </c>
       <c r="D318" s="3" t="n">
-        <v>46272</v>
+        <v>46262</v>
       </c>
       <c r="E318" s="4" t="inlineStr">
         <is>
@@ -26423,9 +26109,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D344" s="3" t="n">
-        <v>46262</v>
-      </c>
+      <c r="D344" s="3" t="n"/>
       <c r="E344" s="4" t="inlineStr">
         <is>
           <t>2630L757</t>
@@ -26497,7 +26181,7 @@
         </is>
       </c>
       <c r="D345" s="3" t="n">
-        <v>46261</v>
+        <v>46256</v>
       </c>
       <c r="E345" s="4" t="inlineStr">
         <is>
@@ -26570,7 +26254,7 @@
         </is>
       </c>
       <c r="D346" s="3" t="n">
-        <v>46261</v>
+        <v>46256</v>
       </c>
       <c r="E346" s="4" t="inlineStr">
         <is>
@@ -26643,7 +26327,7 @@
         </is>
       </c>
       <c r="D347" s="3" t="n">
-        <v>46261</v>
+        <v>46256</v>
       </c>
       <c r="E347" s="4" t="inlineStr">
         <is>
@@ -26716,7 +26400,7 @@
         </is>
       </c>
       <c r="D348" s="3" t="n">
-        <v>46261</v>
+        <v>46256</v>
       </c>
       <c r="E348" s="4" t="inlineStr">
         <is>
@@ -26789,7 +26473,7 @@
         </is>
       </c>
       <c r="D349" s="3" t="n">
-        <v>46261</v>
+        <v>46256</v>
       </c>
       <c r="E349" s="4" t="inlineStr">
         <is>
@@ -26862,7 +26546,7 @@
         </is>
       </c>
       <c r="D350" s="3" t="n">
-        <v>46261</v>
+        <v>46256</v>
       </c>
       <c r="E350" s="4" t="inlineStr">
         <is>
@@ -26935,7 +26619,7 @@
         </is>
       </c>
       <c r="D351" s="3" t="n">
-        <v>46261</v>
+        <v>46256</v>
       </c>
       <c r="E351" s="4" t="inlineStr">
         <is>
@@ -27081,7 +26765,7 @@
         </is>
       </c>
       <c r="D353" s="3" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="E353" s="4" t="inlineStr">
         <is>
@@ -27154,7 +26838,7 @@
         </is>
       </c>
       <c r="D354" s="3" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="E354" s="4" t="inlineStr">
         <is>
@@ -27227,7 +26911,7 @@
         </is>
       </c>
       <c r="D355" s="3" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="E355" s="4" t="inlineStr">
         <is>
@@ -28831,7 +28515,7 @@
         </is>
       </c>
       <c r="D377" s="3" t="n">
-        <v>46268</v>
+        <v>46262</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -28904,7 +28588,7 @@
         </is>
       </c>
       <c r="D378" s="3" t="n">
-        <v>46268</v>
+        <v>46262</v>
       </c>
       <c r="E378" t="inlineStr">
         <is>
@@ -29050,7 +28734,7 @@
         </is>
       </c>
       <c r="D380" s="3" t="n">
-        <v>46268</v>
+        <v>46258</v>
       </c>
       <c r="E380" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Label each lot with the date bucket it is currently paying off
CoveredThroughDate is now the earliest date whose full-day cumulative
demand still exceeds the running supply *before* this lot is added
(next_uncovered_date), rather than the latest date already fully paid
off by supply *after* adding it. A lot that only partly closes a date's
gap is still labeled with that date, and the label only advances once
the running supply (as of the prior lot) has crossed that date's full
total.

Verified against T521B156M025ATE100: lots 1-2 -> 2026-08-22, lots 3-9
-> 2026-08-26, lots 10-11 -> 2026-08-29, matching the manual gap
calculation exactly (396,554.67 / 729,170.18 / 1,669,448.63 minus
PlannedQty and cumulative lot quantities).
</commit_message>
<xml_diff>
--- a/shortage_with_anode_report.xlsx
+++ b/shortage_with_anode_report.xlsx
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1542,7 +1542,7 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1615,7 +1615,7 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1688,7 +1688,7 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1761,7 +1761,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1834,7 +1834,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -2126,7 +2126,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46276</v>
+        <v>46278</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2199,7 +2199,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46276</v>
+        <v>46278</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2272,7 +2272,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46276</v>
+        <v>46278</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2345,7 +2345,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
@@ -2418,7 +2418,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
@@ -2491,7 +2491,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
@@ -2564,7 +2564,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
@@ -2710,7 +2710,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
@@ -2783,7 +2783,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
@@ -2856,7 +2856,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
@@ -3002,7 +3002,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
@@ -3075,7 +3075,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
@@ -3148,7 +3148,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
@@ -3294,7 +3294,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
@@ -3367,7 +3367,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
@@ -3513,7 +3513,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46272</v>
+        <v>46278</v>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
@@ -3586,7 +3586,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46272</v>
+        <v>46278</v>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
@@ -3659,7 +3659,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46272</v>
+        <v>46278</v>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
@@ -3732,7 +3732,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46272</v>
+        <v>46278</v>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
@@ -3805,7 +3805,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46272</v>
+        <v>46278</v>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
@@ -3878,7 +3878,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46272</v>
+        <v>46278</v>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
@@ -4024,7 +4024,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46277</v>
+        <v>46263</v>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
@@ -4096,7 +4096,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D38" s="3" t="n"/>
+      <c r="D38" s="3" t="n">
+        <v>46253</v>
+      </c>
       <c r="E38" t="inlineStr">
         <is>
           <t>2631GZ37</t>
@@ -4167,7 +4169,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D39" s="3" t="n"/>
+      <c r="D39" s="3" t="n">
+        <v>46253</v>
+      </c>
       <c r="E39" t="inlineStr">
         <is>
           <t>2631H237</t>
@@ -4238,7 +4242,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D40" s="3" t="n"/>
+      <c r="D40" s="3" t="n">
+        <v>46253</v>
+      </c>
       <c r="E40" t="inlineStr">
         <is>
           <t>2631KK47</t>
@@ -4309,7 +4315,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D41" s="3" t="n"/>
+      <c r="D41" s="3" t="n">
+        <v>46253</v>
+      </c>
       <c r="E41" t="inlineStr">
         <is>
           <t>2631HN57</t>
@@ -4380,7 +4388,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D42" s="3" t="n"/>
+      <c r="D42" s="3" t="n">
+        <v>46253</v>
+      </c>
       <c r="E42" t="inlineStr">
         <is>
           <t>2631HO27</t>
@@ -4451,7 +4461,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D43" s="3" t="n"/>
+      <c r="D43" s="3" t="n">
+        <v>46253</v>
+      </c>
       <c r="E43" t="inlineStr">
         <is>
           <t>2631KO47</t>
@@ -4522,7 +4534,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D44" s="3" t="n"/>
+      <c r="D44" s="3" t="n">
+        <v>46253</v>
+      </c>
       <c r="E44" t="inlineStr">
         <is>
           <t>2631H137</t>
@@ -4594,7 +4608,7 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46253</v>
+        <v>46258</v>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
@@ -4667,7 +4681,7 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46262</v>
+        <v>46258</v>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
@@ -4740,7 +4754,7 @@
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
@@ -4813,7 +4827,7 @@
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
@@ -4959,7 +4973,7 @@
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
@@ -5032,7 +5046,7 @@
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
@@ -5105,7 +5119,7 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
@@ -5178,7 +5192,7 @@
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
@@ -5251,7 +5265,7 @@
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
@@ -5324,7 +5338,7 @@
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
@@ -5470,7 +5484,7 @@
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>46267</v>
+        <v>46272</v>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
@@ -5543,7 +5557,7 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>46267</v>
+        <v>46272</v>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
@@ -5616,7 +5630,7 @@
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>46267</v>
+        <v>46272</v>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
@@ -5689,7 +5703,7 @@
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>46276</v>
+        <v>46272</v>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
@@ -5762,7 +5776,7 @@
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
@@ -5835,7 +5849,7 @@
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
@@ -5908,7 +5922,7 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
@@ -5981,7 +5995,7 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
@@ -6054,7 +6068,7 @@
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>46279</v>
+        <v>46277</v>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
@@ -6127,7 +6141,7 @@
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>46279</v>
+        <v>46281</v>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
@@ -6199,7 +6213,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="D67" s="3" t="n"/>
+      <c r="D67" s="3" t="n">
+        <v>46256</v>
+      </c>
       <c r="E67" t="inlineStr">
         <is>
           <t>2631GM37</t>
@@ -6344,7 +6360,7 @@
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>46256</v>
+        <v>46260</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -6417,7 +6433,7 @@
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>46256</v>
+        <v>46260</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -6490,7 +6506,7 @@
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>46256</v>
+        <v>46260</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -6563,7 +6579,7 @@
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>46256</v>
+        <v>46260</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -6636,7 +6652,7 @@
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>46256</v>
+        <v>46260</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -6709,7 +6725,7 @@
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>46256</v>
+        <v>46260</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -6855,7 +6871,7 @@
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>46260</v>
+        <v>46263</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -6928,7 +6944,7 @@
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>46260</v>
+        <v>46263</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -7001,7 +7017,7 @@
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -7147,7 +7163,7 @@
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>46261</v>
+        <v>46265</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -7220,7 +7236,7 @@
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>46261</v>
+        <v>46265</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -7293,7 +7309,7 @@
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
@@ -7366,7 +7382,7 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
@@ -7439,7 +7455,7 @@
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
@@ -7512,7 +7528,7 @@
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
@@ -7585,7 +7601,7 @@
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
@@ -7658,7 +7674,7 @@
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E87" s="4" t="inlineStr">
         <is>
@@ -7731,7 +7747,7 @@
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
@@ -7804,7 +7820,7 @@
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
@@ -7877,7 +7893,7 @@
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
@@ -7950,7 +7966,7 @@
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
@@ -8023,7 +8039,7 @@
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
@@ -8096,7 +8112,7 @@
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E93" s="4" t="inlineStr">
         <is>
@@ -8169,7 +8185,7 @@
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
@@ -8242,7 +8258,7 @@
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E95" s="4" t="inlineStr">
         <is>
@@ -8315,7 +8331,7 @@
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
@@ -8388,7 +8404,7 @@
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E97" s="4" t="inlineStr">
         <is>
@@ -8461,7 +8477,7 @@
         </is>
       </c>
       <c r="D98" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
@@ -8534,7 +8550,7 @@
         </is>
       </c>
       <c r="D99" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E99" s="4" t="inlineStr">
         <is>
@@ -8607,7 +8623,7 @@
         </is>
       </c>
       <c r="D100" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
@@ -8680,7 +8696,7 @@
         </is>
       </c>
       <c r="D101" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E101" s="4" t="inlineStr">
         <is>
@@ -8753,7 +8769,7 @@
         </is>
       </c>
       <c r="D102" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
@@ -8826,7 +8842,7 @@
         </is>
       </c>
       <c r="D103" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E103" s="4" t="inlineStr">
         <is>
@@ -8899,7 +8915,7 @@
         </is>
       </c>
       <c r="D104" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
@@ -8972,7 +8988,7 @@
         </is>
       </c>
       <c r="D105" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E105" s="4" t="inlineStr">
         <is>
@@ -9045,7 +9061,7 @@
         </is>
       </c>
       <c r="D106" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
@@ -9191,7 +9207,7 @@
         </is>
       </c>
       <c r="D108" s="3" t="n">
-        <v>46258</v>
+        <v>46268</v>
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
@@ -9264,7 +9280,7 @@
         </is>
       </c>
       <c r="D109" s="3" t="n">
-        <v>46258</v>
+        <v>46268</v>
       </c>
       <c r="E109" s="4" t="inlineStr">
         <is>
@@ -9337,7 +9353,7 @@
         </is>
       </c>
       <c r="D110" s="3" t="n">
-        <v>46258</v>
+        <v>46268</v>
       </c>
       <c r="E110" s="4" t="inlineStr">
         <is>
@@ -9410,7 +9426,7 @@
         </is>
       </c>
       <c r="D111" s="3" t="n">
-        <v>46258</v>
+        <v>46268</v>
       </c>
       <c r="E111" s="4" t="inlineStr">
         <is>
@@ -9556,7 +9572,7 @@
         </is>
       </c>
       <c r="D113" s="3" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="E113" s="4" t="inlineStr">
         <is>
@@ -9702,7 +9718,7 @@
         </is>
       </c>
       <c r="D115" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E115" s="4" t="inlineStr">
         <is>
@@ -9775,7 +9791,7 @@
         </is>
       </c>
       <c r="D116" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
@@ -9848,7 +9864,7 @@
         </is>
       </c>
       <c r="D117" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E117" s="4" t="inlineStr">
         <is>
@@ -9921,7 +9937,7 @@
         </is>
       </c>
       <c r="D118" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
@@ -9994,7 +10010,7 @@
         </is>
       </c>
       <c r="D119" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E119" s="4" t="inlineStr">
         <is>
@@ -10067,7 +10083,7 @@
         </is>
       </c>
       <c r="D120" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
@@ -10140,7 +10156,7 @@
         </is>
       </c>
       <c r="D121" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E121" s="4" t="inlineStr">
         <is>
@@ -10213,7 +10229,7 @@
         </is>
       </c>
       <c r="D122" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
@@ -10286,7 +10302,7 @@
         </is>
       </c>
       <c r="D123" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E123" s="4" t="inlineStr">
         <is>
@@ -10359,7 +10375,7 @@
         </is>
       </c>
       <c r="D124" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E124" s="4" t="inlineStr">
         <is>
@@ -10432,7 +10448,7 @@
         </is>
       </c>
       <c r="D125" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E125" s="4" t="inlineStr">
         <is>
@@ -10505,7 +10521,7 @@
         </is>
       </c>
       <c r="D126" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E126" s="4" t="inlineStr">
         <is>
@@ -10578,7 +10594,7 @@
         </is>
       </c>
       <c r="D127" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E127" s="4" t="inlineStr">
         <is>
@@ -10651,7 +10667,7 @@
         </is>
       </c>
       <c r="D128" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E128" s="4" t="inlineStr">
         <is>
@@ -10724,7 +10740,7 @@
         </is>
       </c>
       <c r="D129" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E129" s="4" t="inlineStr">
         <is>
@@ -10797,7 +10813,7 @@
         </is>
       </c>
       <c r="D130" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E130" s="4" t="inlineStr">
         <is>
@@ -10870,7 +10886,7 @@
         </is>
       </c>
       <c r="D131" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E131" s="4" t="inlineStr">
         <is>
@@ -10943,7 +10959,7 @@
         </is>
       </c>
       <c r="D132" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E132" s="4" t="inlineStr">
         <is>
@@ -11016,7 +11032,7 @@
         </is>
       </c>
       <c r="D133" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E133" s="4" t="inlineStr">
         <is>
@@ -11089,7 +11105,7 @@
         </is>
       </c>
       <c r="D134" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E134" s="4" t="inlineStr">
         <is>
@@ -11162,7 +11178,7 @@
         </is>
       </c>
       <c r="D135" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E135" s="4" t="inlineStr">
         <is>
@@ -11235,7 +11251,7 @@
         </is>
       </c>
       <c r="D136" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E136" s="4" t="inlineStr">
         <is>
@@ -11308,7 +11324,7 @@
         </is>
       </c>
       <c r="D137" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E137" s="4" t="inlineStr">
         <is>
@@ -11381,7 +11397,7 @@
         </is>
       </c>
       <c r="D138" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E138" s="4" t="inlineStr">
         <is>
@@ -11454,7 +11470,7 @@
         </is>
       </c>
       <c r="D139" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E139" s="4" t="inlineStr">
         <is>
@@ -11527,7 +11543,7 @@
         </is>
       </c>
       <c r="D140" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E140" s="4" t="inlineStr">
         <is>
@@ -11600,7 +11616,7 @@
         </is>
       </c>
       <c r="D141" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E141" s="4" t="inlineStr">
         <is>
@@ -11673,7 +11689,7 @@
         </is>
       </c>
       <c r="D142" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E142" s="4" t="inlineStr">
         <is>
@@ -11746,7 +11762,7 @@
         </is>
       </c>
       <c r="D143" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E143" s="4" t="inlineStr">
         <is>
@@ -11819,7 +11835,7 @@
         </is>
       </c>
       <c r="D144" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E144" s="4" t="inlineStr">
         <is>
@@ -11892,7 +11908,7 @@
         </is>
       </c>
       <c r="D145" s="3" t="n">
-        <v>46272</v>
+        <v>46275</v>
       </c>
       <c r="E145" s="4" t="inlineStr">
         <is>
@@ -12038,7 +12054,7 @@
         </is>
       </c>
       <c r="D147" s="3" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="E147" s="4" t="inlineStr">
         <is>
@@ -12111,7 +12127,7 @@
         </is>
       </c>
       <c r="D148" s="3" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
@@ -12184,7 +12200,7 @@
         </is>
       </c>
       <c r="D149" s="3" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="E149" s="4" t="inlineStr">
         <is>
@@ -12330,7 +12346,7 @@
         </is>
       </c>
       <c r="D151" s="3" t="n">
-        <v>46276</v>
+        <v>46282</v>
       </c>
       <c r="E151" s="4" t="inlineStr">
         <is>
@@ -12403,7 +12419,7 @@
         </is>
       </c>
       <c r="D152" s="3" t="n">
-        <v>46276</v>
+        <v>46282</v>
       </c>
       <c r="E152" s="4" t="inlineStr">
         <is>
@@ -12476,7 +12492,7 @@
         </is>
       </c>
       <c r="D153" s="3" t="n">
-        <v>46276</v>
+        <v>46282</v>
       </c>
       <c r="E153" s="4" t="inlineStr">
         <is>
@@ -12549,7 +12565,7 @@
         </is>
       </c>
       <c r="D154" s="3" t="n">
-        <v>46276</v>
+        <v>46282</v>
       </c>
       <c r="E154" s="4" t="inlineStr">
         <is>
@@ -12621,7 +12637,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D155" s="3" t="n"/>
+      <c r="D155" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E155" s="4" t="inlineStr">
         <is>
           <t>2629UT37</t>
@@ -12692,7 +12710,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D156" s="3" t="n"/>
+      <c r="D156" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
           <t>2629LK57</t>
@@ -12763,7 +12783,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D157" s="3" t="n"/>
+      <c r="D157" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E157" s="4" t="inlineStr">
         <is>
           <t>2630OC17</t>
@@ -12834,7 +12856,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D158" s="3" t="n"/>
+      <c r="D158" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E158" s="4" t="inlineStr">
         <is>
           <t>2630SW37</t>
@@ -12905,7 +12929,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D159" s="3" t="n"/>
+      <c r="D159" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E159" s="4" t="inlineStr">
         <is>
           <t>2630SQ37</t>
@@ -12976,7 +13002,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D160" s="3" t="n"/>
+      <c r="D160" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
           <t>2630S447</t>
@@ -13047,7 +13075,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D161" s="3" t="n"/>
+      <c r="D161" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E161" s="4" t="inlineStr">
         <is>
           <t>2630QV47</t>
@@ -13118,7 +13148,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D162" s="3" t="n"/>
+      <c r="D162" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
           <t>2630S747</t>
@@ -13189,7 +13221,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D163" s="3" t="n"/>
+      <c r="D163" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E163" s="4" t="inlineStr">
         <is>
           <t>2630QY47</t>
@@ -13260,7 +13294,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D164" s="3" t="n"/>
+      <c r="D164" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
           <t>2630OB67</t>
@@ -13331,7 +13367,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D165" s="3" t="n"/>
+      <c r="D165" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E165" s="4" t="inlineStr">
         <is>
           <t>2631P427</t>
@@ -13402,7 +13440,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D166" s="3" t="n"/>
+      <c r="D166" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
           <t>2630O867</t>
@@ -13473,7 +13513,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D167" s="3" t="n"/>
+      <c r="D167" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E167" s="4" t="inlineStr">
         <is>
           <t>2630O967</t>
@@ -13544,7 +13586,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D168" s="3" t="n"/>
+      <c r="D168" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
           <t>2630OA67</t>
@@ -13615,7 +13659,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D169" s="3" t="n"/>
+      <c r="D169" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E169" s="4" t="inlineStr">
         <is>
           <t>2630OC67</t>
@@ -13686,7 +13732,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D170" s="3" t="n"/>
+      <c r="D170" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
           <t>2630OE67</t>
@@ -13757,7 +13805,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D171" s="3" t="n"/>
+      <c r="D171" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E171" s="4" t="inlineStr">
         <is>
           <t>2630OF67</t>
@@ -13828,7 +13878,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D172" s="3" t="n"/>
+      <c r="D172" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
           <t>2630OG67</t>
@@ -13899,7 +13951,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D173" s="3" t="n"/>
+      <c r="D173" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E173" s="4" t="inlineStr">
         <is>
           <t>2631ID17</t>
@@ -13970,7 +14024,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D174" s="3" t="n"/>
+      <c r="D174" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
           <t>2631IE17</t>
@@ -14041,7 +14097,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D175" s="3" t="n"/>
+      <c r="D175" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E175" s="4" t="inlineStr">
         <is>
           <t>2631IF17</t>
@@ -14112,7 +14170,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D176" s="3" t="n"/>
+      <c r="D176" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
           <t>2631IG17</t>
@@ -14183,7 +14243,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D177" s="3" t="n"/>
+      <c r="D177" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E177" s="4" t="inlineStr">
         <is>
           <t>2631IH17</t>
@@ -14254,7 +14316,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D178" s="3" t="n"/>
+      <c r="D178" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E178" s="4" t="inlineStr">
         <is>
           <t>2631II17</t>
@@ -14325,7 +14389,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D179" s="3" t="n"/>
+      <c r="D179" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
           <t>2631IJ17</t>
@@ -14396,7 +14462,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D180" s="3" t="n"/>
+      <c r="D180" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E180" s="4" t="inlineStr">
         <is>
           <t>2631IK17</t>
@@ -14467,7 +14535,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D181" s="3" t="n"/>
+      <c r="D181" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
           <t>2631OW27</t>
@@ -14538,7 +14608,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D182" s="3" t="n"/>
+      <c r="D182" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E182" s="4" t="inlineStr">
         <is>
           <t>2631OX27</t>
@@ -14609,7 +14681,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D183" s="3" t="n"/>
+      <c r="D183" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
           <t>2631OY27</t>
@@ -14680,7 +14754,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D184" s="3" t="n"/>
+      <c r="D184" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E184" s="4" t="inlineStr">
         <is>
           <t>2631OZ27</t>
@@ -14751,7 +14827,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D185" s="3" t="n"/>
+      <c r="D185" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
           <t>2631P327</t>
@@ -14822,7 +14900,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D186" s="3" t="n"/>
+      <c r="D186" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E186" s="4" t="inlineStr">
         <is>
           <t>2631P127</t>
@@ -14893,7 +14973,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D187" s="3" t="n"/>
+      <c r="D187" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
           <t>2631L237</t>
@@ -14964,7 +15046,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D188" s="3" t="n"/>
+      <c r="D188" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E188" s="4" t="inlineStr">
         <is>
           <t>2631L337</t>
@@ -15035,7 +15119,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D189" s="3" t="n"/>
+      <c r="D189" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
           <t>2631L437</t>
@@ -15106,7 +15192,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D190" s="3" t="n"/>
+      <c r="D190" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E190" s="4" t="inlineStr">
         <is>
           <t>2631OV27</t>
@@ -15177,7 +15265,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D191" s="3" t="n"/>
+      <c r="D191" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
           <t>2631P227</t>
@@ -15248,7 +15338,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D192" s="3" t="n"/>
+      <c r="D192" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E192" s="4" t="inlineStr">
         <is>
           <t>2631P627</t>
@@ -15319,7 +15411,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D193" s="3" t="n"/>
+      <c r="D193" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
           <t>2631KS37</t>
@@ -15390,7 +15484,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D194" s="3" t="n"/>
+      <c r="D194" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E194" s="4" t="inlineStr">
         <is>
           <t>2631KZ37</t>
@@ -15461,7 +15557,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D195" s="3" t="n"/>
+      <c r="D195" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
           <t>2631L137</t>
@@ -15532,7 +15630,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D196" s="3" t="n"/>
+      <c r="D196" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E196" s="4" t="inlineStr">
         <is>
           <t>2631P727</t>
@@ -15603,7 +15703,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D197" s="3" t="n"/>
+      <c r="D197" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
           <t>2631KT37</t>
@@ -15674,7 +15776,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D198" s="3" t="n"/>
+      <c r="D198" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E198" s="4" t="inlineStr">
         <is>
           <t>2631KU37</t>
@@ -15745,7 +15849,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D199" s="3" t="n"/>
+      <c r="D199" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
           <t>2631KV37</t>
@@ -15816,7 +15922,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D200" s="3" t="n"/>
+      <c r="D200" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E200" s="4" t="inlineStr">
         <is>
           <t>2631KW37</t>
@@ -15887,7 +15995,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D201" s="3" t="n"/>
+      <c r="D201" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
           <t>2631KX37</t>
@@ -15958,7 +16068,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D202" s="3" t="n"/>
+      <c r="D202" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E202" s="4" t="inlineStr">
         <is>
           <t>2631PW47</t>
@@ -16029,7 +16141,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D203" s="3" t="n"/>
+      <c r="D203" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
           <t>2631PZ47</t>
@@ -16100,7 +16214,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D204" s="3" t="n"/>
+      <c r="D204" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E204" s="4" t="inlineStr">
         <is>
           <t>2631Q147</t>
@@ -16171,7 +16287,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D205" s="3" t="n"/>
+      <c r="D205" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E205" s="4" t="inlineStr">
         <is>
           <t>2631KY37</t>
@@ -16242,7 +16360,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D206" s="3" t="n"/>
+      <c r="D206" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E206" s="4" t="inlineStr">
         <is>
           <t>2631P527</t>
@@ -16313,7 +16433,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D207" s="3" t="n"/>
+      <c r="D207" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E207" s="4" t="inlineStr">
         <is>
           <t>2631KR37</t>
@@ -16384,7 +16506,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D208" s="3" t="n"/>
+      <c r="D208" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E208" s="4" t="inlineStr">
         <is>
           <t>2631L537</t>
@@ -16455,7 +16579,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D209" s="3" t="n"/>
+      <c r="D209" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E209" s="4" t="inlineStr">
         <is>
           <t>2631L637</t>
@@ -16526,7 +16652,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D210" s="3" t="n"/>
+      <c r="D210" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E210" s="4" t="inlineStr">
         <is>
           <t>2631PX47</t>
@@ -16597,7 +16725,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D211" s="3" t="n"/>
+      <c r="D211" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E211" s="4" t="inlineStr">
         <is>
           <t>2631PY47</t>
@@ -16668,7 +16798,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D212" s="3" t="n"/>
+      <c r="D212" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E212" s="4" t="inlineStr">
         <is>
           <t>2631Q347</t>
@@ -16739,7 +16871,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D213" s="3" t="n"/>
+      <c r="D213" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E213" s="4" t="inlineStr">
         <is>
           <t>2631OJ57</t>
@@ -16810,7 +16944,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D214" s="3" t="n"/>
+      <c r="D214" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E214" s="4" t="inlineStr">
         <is>
           <t>2631OL57</t>
@@ -16881,7 +17017,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D215" s="3" t="n"/>
+      <c r="D215" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E215" s="4" t="inlineStr">
         <is>
           <t>2631ON57</t>
@@ -16952,7 +17090,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D216" s="3" t="n"/>
+      <c r="D216" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E216" s="4" t="inlineStr">
         <is>
           <t>2631FZ67</t>
@@ -17023,7 +17163,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D217" s="3" t="n"/>
+      <c r="D217" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E217" s="4" t="inlineStr">
         <is>
           <t>2631G767</t>
@@ -17094,7 +17236,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D218" s="3" t="n"/>
+      <c r="D218" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E218" s="4" t="inlineStr">
         <is>
           <t>2631Q247</t>
@@ -17165,7 +17309,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D219" s="3" t="n"/>
+      <c r="D219" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E219" s="4" t="inlineStr">
         <is>
           <t>2631Q547</t>
@@ -17236,7 +17382,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D220" s="3" t="n"/>
+      <c r="D220" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E220" s="4" t="inlineStr">
         <is>
           <t>2631OI57</t>
@@ -17307,7 +17455,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D221" s="3" t="n"/>
+      <c r="D221" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E221" s="4" t="inlineStr">
         <is>
           <t>2631OM57</t>
@@ -17378,7 +17528,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D222" s="3" t="n"/>
+      <c r="D222" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E222" s="4" t="inlineStr">
         <is>
           <t>2631OO57</t>
@@ -17449,7 +17601,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D223" s="3" t="n"/>
+      <c r="D223" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E223" s="4" t="inlineStr">
         <is>
           <t>2631G367</t>
@@ -17520,7 +17674,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D224" s="3" t="n"/>
+      <c r="D224" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E224" s="4" t="inlineStr">
         <is>
           <t>2631G467</t>
@@ -17591,7 +17747,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D225" s="3" t="n"/>
+      <c r="D225" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E225" s="4" t="inlineStr">
         <is>
           <t>2631Q447</t>
@@ -17662,7 +17820,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D226" s="3" t="n"/>
+      <c r="D226" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E226" s="4" t="inlineStr">
         <is>
           <t>2631OK57</t>
@@ -17733,7 +17893,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D227" s="3" t="n"/>
+      <c r="D227" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E227" s="4" t="inlineStr">
         <is>
           <t>2631FY67</t>
@@ -17804,7 +17966,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D228" s="3" t="n"/>
+      <c r="D228" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E228" s="4" t="inlineStr">
         <is>
           <t>2629UT37</t>
@@ -17875,7 +18039,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D229" s="3" t="n"/>
+      <c r="D229" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E229" s="4" t="inlineStr">
         <is>
           <t>2629LK57</t>
@@ -17946,7 +18112,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D230" s="3" t="n"/>
+      <c r="D230" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E230" s="4" t="inlineStr">
         <is>
           <t>2630OC17</t>
@@ -18017,7 +18185,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D231" s="3" t="n"/>
+      <c r="D231" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E231" s="4" t="inlineStr">
         <is>
           <t>2630SW37</t>
@@ -18088,7 +18258,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D232" s="3" t="n"/>
+      <c r="D232" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E232" s="4" t="inlineStr">
         <is>
           <t>2630SQ37</t>
@@ -18159,7 +18331,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D233" s="3" t="n"/>
+      <c r="D233" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E233" s="4" t="inlineStr">
         <is>
           <t>2630S447</t>
@@ -18230,7 +18404,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D234" s="3" t="n"/>
+      <c r="D234" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E234" s="4" t="inlineStr">
         <is>
           <t>2630QV47</t>
@@ -18301,7 +18477,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D235" s="3" t="n"/>
+      <c r="D235" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E235" s="4" t="inlineStr">
         <is>
           <t>2630S747</t>
@@ -18372,7 +18550,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D236" s="3" t="n"/>
+      <c r="D236" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E236" s="4" t="inlineStr">
         <is>
           <t>2630QY47</t>
@@ -18443,7 +18623,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D237" s="3" t="n"/>
+      <c r="D237" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E237" s="4" t="inlineStr">
         <is>
           <t>2630OB67</t>
@@ -18514,7 +18696,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D238" s="3" t="n"/>
+      <c r="D238" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E238" s="4" t="inlineStr">
         <is>
           <t>2631P427</t>
@@ -18585,7 +18769,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D239" s="3" t="n"/>
+      <c r="D239" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E239" s="4" t="inlineStr">
         <is>
           <t>2630O867</t>
@@ -18656,7 +18842,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D240" s="3" t="n"/>
+      <c r="D240" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E240" s="4" t="inlineStr">
         <is>
           <t>2630O967</t>
@@ -18727,7 +18915,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D241" s="3" t="n"/>
+      <c r="D241" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E241" s="4" t="inlineStr">
         <is>
           <t>2630OA67</t>
@@ -18798,7 +18988,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D242" s="3" t="n"/>
+      <c r="D242" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E242" s="4" t="inlineStr">
         <is>
           <t>2630OC67</t>
@@ -18869,7 +19061,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D243" s="3" t="n"/>
+      <c r="D243" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E243" s="4" t="inlineStr">
         <is>
           <t>2630OE67</t>
@@ -18940,7 +19134,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D244" s="3" t="n"/>
+      <c r="D244" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E244" s="4" t="inlineStr">
         <is>
           <t>2630OF67</t>
@@ -19011,7 +19207,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D245" s="3" t="n"/>
+      <c r="D245" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E245" s="4" t="inlineStr">
         <is>
           <t>2630OG67</t>
@@ -19082,7 +19280,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D246" s="3" t="n"/>
+      <c r="D246" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E246" s="4" t="inlineStr">
         <is>
           <t>2631ID17</t>
@@ -19153,7 +19353,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D247" s="3" t="n"/>
+      <c r="D247" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E247" s="4" t="inlineStr">
         <is>
           <t>2631IE17</t>
@@ -19224,7 +19426,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D248" s="3" t="n"/>
+      <c r="D248" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E248" s="4" t="inlineStr">
         <is>
           <t>2631IF17</t>
@@ -19295,7 +19499,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D249" s="3" t="n"/>
+      <c r="D249" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E249" s="4" t="inlineStr">
         <is>
           <t>2631IG17</t>
@@ -19366,7 +19572,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D250" s="3" t="n"/>
+      <c r="D250" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E250" s="4" t="inlineStr">
         <is>
           <t>2631IH17</t>
@@ -19437,7 +19645,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D251" s="3" t="n"/>
+      <c r="D251" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E251" s="4" t="inlineStr">
         <is>
           <t>2631II17</t>
@@ -19508,7 +19718,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D252" s="3" t="n"/>
+      <c r="D252" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E252" s="4" t="inlineStr">
         <is>
           <t>2631IJ17</t>
@@ -19579,7 +19791,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D253" s="3" t="n"/>
+      <c r="D253" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E253" s="4" t="inlineStr">
         <is>
           <t>2631IK17</t>
@@ -19650,7 +19864,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D254" s="3" t="n"/>
+      <c r="D254" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E254" s="4" t="inlineStr">
         <is>
           <t>2631OW27</t>
@@ -19721,7 +19937,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D255" s="3" t="n"/>
+      <c r="D255" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E255" s="4" t="inlineStr">
         <is>
           <t>2631OX27</t>
@@ -19792,7 +20010,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D256" s="3" t="n"/>
+      <c r="D256" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E256" s="4" t="inlineStr">
         <is>
           <t>2631OY27</t>
@@ -19863,7 +20083,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D257" s="3" t="n"/>
+      <c r="D257" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E257" s="4" t="inlineStr">
         <is>
           <t>2631OZ27</t>
@@ -19934,7 +20156,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D258" s="3" t="n"/>
+      <c r="D258" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E258" s="4" t="inlineStr">
         <is>
           <t>2631P327</t>
@@ -20005,7 +20229,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D259" s="3" t="n"/>
+      <c r="D259" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E259" s="4" t="inlineStr">
         <is>
           <t>2631P127</t>
@@ -20076,7 +20302,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D260" s="3" t="n"/>
+      <c r="D260" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E260" s="4" t="inlineStr">
         <is>
           <t>2631L237</t>
@@ -20147,7 +20375,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D261" s="3" t="n"/>
+      <c r="D261" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E261" s="4" t="inlineStr">
         <is>
           <t>2631L337</t>
@@ -20218,7 +20448,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D262" s="3" t="n"/>
+      <c r="D262" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E262" s="4" t="inlineStr">
         <is>
           <t>2631L437</t>
@@ -20289,7 +20521,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D263" s="3" t="n"/>
+      <c r="D263" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E263" s="4" t="inlineStr">
         <is>
           <t>2631OV27</t>
@@ -20360,7 +20594,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D264" s="3" t="n"/>
+      <c r="D264" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E264" s="4" t="inlineStr">
         <is>
           <t>2631P227</t>
@@ -20431,7 +20667,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D265" s="3" t="n"/>
+      <c r="D265" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E265" s="4" t="inlineStr">
         <is>
           <t>2631P627</t>
@@ -20502,7 +20740,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D266" s="3" t="n"/>
+      <c r="D266" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E266" s="4" t="inlineStr">
         <is>
           <t>2631KS37</t>
@@ -20573,7 +20813,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D267" s="3" t="n"/>
+      <c r="D267" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E267" s="4" t="inlineStr">
         <is>
           <t>2631KZ37</t>
@@ -20644,7 +20886,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D268" s="3" t="n"/>
+      <c r="D268" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E268" s="4" t="inlineStr">
         <is>
           <t>2631L137</t>
@@ -20715,7 +20959,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D269" s="3" t="n"/>
+      <c r="D269" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E269" s="4" t="inlineStr">
         <is>
           <t>2631P727</t>
@@ -20786,7 +21032,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D270" s="3" t="n"/>
+      <c r="D270" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E270" s="4" t="inlineStr">
         <is>
           <t>2631KT37</t>
@@ -20857,7 +21105,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D271" s="3" t="n"/>
+      <c r="D271" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E271" s="4" t="inlineStr">
         <is>
           <t>2631KU37</t>
@@ -20928,7 +21178,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D272" s="3" t="n"/>
+      <c r="D272" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E272" s="4" t="inlineStr">
         <is>
           <t>2631KV37</t>
@@ -20999,7 +21251,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D273" s="3" t="n"/>
+      <c r="D273" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E273" s="4" t="inlineStr">
         <is>
           <t>2631KW37</t>
@@ -21070,7 +21324,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D274" s="3" t="n"/>
+      <c r="D274" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E274" s="4" t="inlineStr">
         <is>
           <t>2631KX37</t>
@@ -21141,7 +21397,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D275" s="3" t="n"/>
+      <c r="D275" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E275" s="4" t="inlineStr">
         <is>
           <t>2631PW47</t>
@@ -21212,7 +21470,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D276" s="3" t="n"/>
+      <c r="D276" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E276" s="4" t="inlineStr">
         <is>
           <t>2631PZ47</t>
@@ -21283,7 +21543,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D277" s="3" t="n"/>
+      <c r="D277" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E277" s="4" t="inlineStr">
         <is>
           <t>2631Q147</t>
@@ -21354,7 +21616,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D278" s="3" t="n"/>
+      <c r="D278" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E278" s="4" t="inlineStr">
         <is>
           <t>2631KY37</t>
@@ -21425,7 +21689,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D279" s="3" t="n"/>
+      <c r="D279" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E279" s="4" t="inlineStr">
         <is>
           <t>2631P527</t>
@@ -21496,7 +21762,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D280" s="3" t="n"/>
+      <c r="D280" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E280" s="4" t="inlineStr">
         <is>
           <t>2631KR37</t>
@@ -21567,7 +21835,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D281" s="3" t="n"/>
+      <c r="D281" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E281" s="4" t="inlineStr">
         <is>
           <t>2631L537</t>
@@ -21638,7 +21908,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D282" s="3" t="n"/>
+      <c r="D282" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E282" s="4" t="inlineStr">
         <is>
           <t>2631L637</t>
@@ -21709,7 +21981,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D283" s="3" t="n"/>
+      <c r="D283" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E283" s="4" t="inlineStr">
         <is>
           <t>2631PX47</t>
@@ -21780,7 +22054,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D284" s="3" t="n"/>
+      <c r="D284" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E284" s="4" t="inlineStr">
         <is>
           <t>2631PY47</t>
@@ -21851,7 +22127,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D285" s="3" t="n"/>
+      <c r="D285" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E285" s="4" t="inlineStr">
         <is>
           <t>2631Q347</t>
@@ -21922,7 +22200,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D286" s="3" t="n"/>
+      <c r="D286" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E286" s="4" t="inlineStr">
         <is>
           <t>2631OJ57</t>
@@ -21993,7 +22273,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D287" s="3" t="n"/>
+      <c r="D287" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E287" s="4" t="inlineStr">
         <is>
           <t>2631OL57</t>
@@ -22064,7 +22346,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D288" s="3" t="n"/>
+      <c r="D288" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E288" s="4" t="inlineStr">
         <is>
           <t>2631ON57</t>
@@ -22135,7 +22419,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D289" s="3" t="n"/>
+      <c r="D289" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E289" s="4" t="inlineStr">
         <is>
           <t>2631FZ67</t>
@@ -22206,7 +22492,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D290" s="3" t="n"/>
+      <c r="D290" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E290" s="4" t="inlineStr">
         <is>
           <t>2631G767</t>
@@ -22277,7 +22565,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D291" s="3" t="n"/>
+      <c r="D291" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E291" s="4" t="inlineStr">
         <is>
           <t>2631Q247</t>
@@ -22348,7 +22638,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D292" s="3" t="n"/>
+      <c r="D292" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E292" s="4" t="inlineStr">
         <is>
           <t>2631Q547</t>
@@ -22419,7 +22711,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D293" s="3" t="n"/>
+      <c r="D293" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E293" s="4" t="inlineStr">
         <is>
           <t>2631OI57</t>
@@ -22490,7 +22784,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D294" s="3" t="n"/>
+      <c r="D294" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E294" s="4" t="inlineStr">
         <is>
           <t>2631OM57</t>
@@ -22561,7 +22857,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D295" s="3" t="n"/>
+      <c r="D295" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E295" s="4" t="inlineStr">
         <is>
           <t>2631OO57</t>
@@ -22632,7 +22930,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D296" s="3" t="n"/>
+      <c r="D296" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E296" s="4" t="inlineStr">
         <is>
           <t>2631G367</t>
@@ -22703,7 +23003,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D297" s="3" t="n"/>
+      <c r="D297" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E297" s="4" t="inlineStr">
         <is>
           <t>2631G467</t>
@@ -22774,7 +23076,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D298" s="3" t="n"/>
+      <c r="D298" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E298" s="4" t="inlineStr">
         <is>
           <t>2631Q447</t>
@@ -22845,7 +23149,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D299" s="3" t="n"/>
+      <c r="D299" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E299" s="4" t="inlineStr">
         <is>
           <t>2631OK57</t>
@@ -22916,7 +23222,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D300" s="3" t="n"/>
+      <c r="D300" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E300" s="4" t="inlineStr">
         <is>
           <t>2631FY67</t>
@@ -22987,7 +23295,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D301" s="3" t="n"/>
+      <c r="D301" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E301" t="inlineStr">
         <is>
           <t>2627FS10</t>
@@ -23058,7 +23368,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D302" s="3" t="n"/>
+      <c r="D302" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E302" t="inlineStr">
         <is>
           <t>2627FR90</t>
@@ -23129,7 +23441,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D303" s="3" t="n"/>
+      <c r="D303" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E303" t="inlineStr">
         <is>
           <t>2627FS20</t>
@@ -23200,7 +23514,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D304" s="3" t="n"/>
+      <c r="D304" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E304" t="inlineStr">
         <is>
           <t>2628FU10</t>
@@ -23271,7 +23587,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D305" s="3" t="n"/>
+      <c r="D305" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E305" t="inlineStr">
         <is>
           <t>2630FY20</t>
@@ -23342,7 +23660,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D306" s="3" t="n"/>
+      <c r="D306" s="3" t="n">
+        <v>46258</v>
+      </c>
       <c r="E306" t="inlineStr">
         <is>
           <t>2630FY30</t>
@@ -23487,7 +23807,7 @@
         </is>
       </c>
       <c r="D308" s="3" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="E308" s="4" t="inlineStr">
         <is>
@@ -23560,7 +23880,7 @@
         </is>
       </c>
       <c r="D309" s="3" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="E309" s="4" t="inlineStr">
         <is>
@@ -23633,7 +23953,7 @@
         </is>
       </c>
       <c r="D310" s="3" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="E310" s="4" t="inlineStr">
         <is>
@@ -23706,7 +24026,7 @@
         </is>
       </c>
       <c r="D311" s="3" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="E311" s="4" t="inlineStr">
         <is>
@@ -23779,7 +24099,7 @@
         </is>
       </c>
       <c r="D312" s="3" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="E312" s="4" t="inlineStr">
         <is>
@@ -23852,7 +24172,7 @@
         </is>
       </c>
       <c r="D313" s="3" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="E313" s="4" t="inlineStr">
         <is>
@@ -23925,7 +24245,7 @@
         </is>
       </c>
       <c r="D314" s="3" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="E314" s="4" t="inlineStr">
         <is>
@@ -23998,7 +24318,7 @@
         </is>
       </c>
       <c r="D315" s="3" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="E315" s="4" t="inlineStr">
         <is>
@@ -24144,7 +24464,7 @@
         </is>
       </c>
       <c r="D317" s="3" t="n">
-        <v>46262</v>
+        <v>46272</v>
       </c>
       <c r="E317" s="4" t="inlineStr">
         <is>
@@ -24217,7 +24537,7 @@
         </is>
       </c>
       <c r="D318" s="3" t="n">
-        <v>46262</v>
+        <v>46272</v>
       </c>
       <c r="E318" s="4" t="inlineStr">
         <is>
@@ -24290,7 +24610,7 @@
         </is>
       </c>
       <c r="D319" s="3" t="n">
-        <v>46279</v>
+        <v>46271</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -24363,7 +24683,7 @@
         </is>
       </c>
       <c r="D320" s="3" t="n">
-        <v>46279</v>
+        <v>46281</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -24431,7 +24751,7 @@
         </is>
       </c>
       <c r="D321" s="3" t="n">
-        <v>46279</v>
+        <v>46281</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -24504,7 +24824,7 @@
         </is>
       </c>
       <c r="D322" s="3" t="n">
-        <v>46279</v>
+        <v>46281</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -24577,7 +24897,7 @@
         </is>
       </c>
       <c r="D323" s="3" t="n">
-        <v>46279</v>
+        <v>46281</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -24650,7 +24970,7 @@
         </is>
       </c>
       <c r="D324" s="3" t="n">
-        <v>46279</v>
+        <v>46281</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -24723,7 +25043,7 @@
         </is>
       </c>
       <c r="D325" s="3" t="n">
-        <v>46279</v>
+        <v>46281</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -24796,7 +25116,7 @@
         </is>
       </c>
       <c r="D326" s="3" t="n">
-        <v>46287</v>
+        <v>46281</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -24868,9 +25188,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D327" s="3" t="n">
-        <v>46287</v>
-      </c>
+      <c r="D327" s="3" t="n"/>
       <c r="E327" t="inlineStr">
         <is>
           <t>2630GA20</t>
@@ -24941,9 +25259,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D328" s="3" t="n">
-        <v>46287</v>
-      </c>
+      <c r="D328" s="3" t="n"/>
       <c r="E328" t="inlineStr">
         <is>
           <t>2630FZ70</t>
@@ -25014,9 +25330,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D329" s="3" t="n">
-        <v>46287</v>
-      </c>
+      <c r="D329" s="3" t="n"/>
       <c r="E329" t="inlineStr">
         <is>
           <t>2630FZ90</t>
@@ -25087,9 +25401,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D330" s="3" t="n">
-        <v>46287</v>
-      </c>
+      <c r="D330" s="3" t="n"/>
       <c r="E330" t="inlineStr">
         <is>
           <t>2630GA30</t>
@@ -25160,9 +25472,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D331" s="3" t="n">
-        <v>46287</v>
-      </c>
+      <c r="D331" s="3" t="n"/>
       <c r="E331" t="inlineStr">
         <is>
           <t>2630GA10</t>
@@ -25233,9 +25543,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D332" s="3" t="n">
-        <v>46287</v>
-      </c>
+      <c r="D332" s="3" t="n"/>
       <c r="E332" t="inlineStr">
         <is>
           <t>2630GB10</t>
@@ -25306,9 +25614,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D333" s="3" t="n">
-        <v>46287</v>
-      </c>
+      <c r="D333" s="3" t="n"/>
       <c r="E333" t="inlineStr">
         <is>
           <t>2630GA90</t>
@@ -25379,9 +25685,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D334" s="3" t="n">
-        <v>46287</v>
-      </c>
+      <c r="D334" s="3" t="n"/>
       <c r="E334" t="inlineStr">
         <is>
           <t>2630GA80</t>
@@ -25452,9 +25756,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D335" s="3" t="n">
-        <v>46287</v>
-      </c>
+      <c r="D335" s="3" t="n"/>
       <c r="E335" t="inlineStr">
         <is>
           <t>2630GB20</t>
@@ -25525,9 +25827,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D336" s="3" t="n">
-        <v>46287</v>
-      </c>
+      <c r="D336" s="3" t="n"/>
       <c r="E336" t="inlineStr">
         <is>
           <t>2630GB40</t>
@@ -25598,9 +25898,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D337" s="3" t="n">
-        <v>46287</v>
-      </c>
+      <c r="D337" s="3" t="n"/>
       <c r="E337" t="inlineStr">
         <is>
           <t>2630GC30</t>
@@ -25671,9 +25969,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D338" s="3" t="n">
-        <v>46287</v>
-      </c>
+      <c r="D338" s="3" t="n"/>
       <c r="E338" t="inlineStr">
         <is>
           <t>2630GB30</t>
@@ -25744,9 +26040,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D339" s="3" t="n">
-        <v>46287</v>
-      </c>
+      <c r="D339" s="3" t="n"/>
       <c r="E339" t="inlineStr">
         <is>
           <t>2630GC50</t>
@@ -25817,9 +26111,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D340" s="3" t="n">
-        <v>46287</v>
-      </c>
+      <c r="D340" s="3" t="n"/>
       <c r="E340" t="inlineStr">
         <is>
           <t>2630GB90</t>
@@ -25890,9 +26182,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D341" s="3" t="n">
-        <v>46287</v>
-      </c>
+      <c r="D341" s="3" t="n"/>
       <c r="E341" t="inlineStr">
         <is>
           <t>2630GC20</t>
@@ -25963,9 +26253,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D342" s="3" t="n">
-        <v>46287</v>
-      </c>
+      <c r="D342" s="3" t="n"/>
       <c r="E342" t="inlineStr">
         <is>
           <t>2630GC10</t>
@@ -26036,9 +26324,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D343" s="3" t="n">
-        <v>46287</v>
-      </c>
+      <c r="D343" s="3" t="n"/>
       <c r="E343" t="inlineStr">
         <is>
           <t>2630GC40</t>
@@ -26109,7 +26395,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D344" s="3" t="n"/>
+      <c r="D344" s="3" t="n">
+        <v>46262</v>
+      </c>
       <c r="E344" s="4" t="inlineStr">
         <is>
           <t>2630L757</t>
@@ -26181,7 +26469,7 @@
         </is>
       </c>
       <c r="D345" s="3" t="n">
-        <v>46256</v>
+        <v>46261</v>
       </c>
       <c r="E345" s="4" t="inlineStr">
         <is>
@@ -26254,7 +26542,7 @@
         </is>
       </c>
       <c r="D346" s="3" t="n">
-        <v>46256</v>
+        <v>46261</v>
       </c>
       <c r="E346" s="4" t="inlineStr">
         <is>
@@ -26327,7 +26615,7 @@
         </is>
       </c>
       <c r="D347" s="3" t="n">
-        <v>46256</v>
+        <v>46261</v>
       </c>
       <c r="E347" s="4" t="inlineStr">
         <is>
@@ -26400,7 +26688,7 @@
         </is>
       </c>
       <c r="D348" s="3" t="n">
-        <v>46256</v>
+        <v>46261</v>
       </c>
       <c r="E348" s="4" t="inlineStr">
         <is>
@@ -26473,7 +26761,7 @@
         </is>
       </c>
       <c r="D349" s="3" t="n">
-        <v>46256</v>
+        <v>46261</v>
       </c>
       <c r="E349" s="4" t="inlineStr">
         <is>
@@ -26546,7 +26834,7 @@
         </is>
       </c>
       <c r="D350" s="3" t="n">
-        <v>46256</v>
+        <v>46261</v>
       </c>
       <c r="E350" s="4" t="inlineStr">
         <is>
@@ -26619,7 +26907,7 @@
         </is>
       </c>
       <c r="D351" s="3" t="n">
-        <v>46256</v>
+        <v>46261</v>
       </c>
       <c r="E351" s="4" t="inlineStr">
         <is>
@@ -26692,7 +26980,7 @@
         </is>
       </c>
       <c r="D352" s="3" t="n">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="E352" s="4" t="inlineStr">
         <is>
@@ -26765,7 +27053,7 @@
         </is>
       </c>
       <c r="D353" s="3" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="E353" s="4" t="inlineStr">
         <is>
@@ -26838,7 +27126,7 @@
         </is>
       </c>
       <c r="D354" s="3" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="E354" s="4" t="inlineStr">
         <is>
@@ -26911,7 +27199,7 @@
         </is>
       </c>
       <c r="D355" s="3" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="E355" s="4" t="inlineStr">
         <is>
@@ -27056,9 +27344,7 @@
           <t>P</t>
         </is>
       </c>
-      <c r="D357" s="3" t="n">
-        <v>46264</v>
-      </c>
+      <c r="D357" s="3" t="n"/>
       <c r="E357" s="4" t="inlineStr">
         <is>
           <t>2623P237</t>
@@ -27129,9 +27415,7 @@
           <t>P</t>
         </is>
       </c>
-      <c r="D358" s="3" t="n">
-        <v>46264</v>
-      </c>
+      <c r="D358" s="3" t="n"/>
       <c r="E358" s="4" t="inlineStr">
         <is>
           <t>2624OF37</t>
@@ -27202,9 +27486,7 @@
           <t>P</t>
         </is>
       </c>
-      <c r="D359" s="3" t="n">
-        <v>46264</v>
-      </c>
+      <c r="D359" s="3" t="n"/>
       <c r="E359" s="4" t="inlineStr">
         <is>
           <t>2624KP57</t>
@@ -27275,9 +27557,7 @@
           <t>P</t>
         </is>
       </c>
-      <c r="D360" s="3" t="n">
-        <v>46264</v>
-      </c>
+      <c r="D360" s="3" t="n"/>
       <c r="E360" s="4" t="inlineStr">
         <is>
           <t>2631HT17</t>
@@ -27348,9 +27628,7 @@
           <t>P</t>
         </is>
       </c>
-      <c r="D361" s="3" t="n">
-        <v>46264</v>
-      </c>
+      <c r="D361" s="3" t="n"/>
       <c r="E361" s="4" t="inlineStr">
         <is>
           <t>2631HU17</t>
@@ -27421,9 +27699,7 @@
           <t>P</t>
         </is>
       </c>
-      <c r="D362" s="3" t="n">
-        <v>46264</v>
-      </c>
+      <c r="D362" s="3" t="n"/>
       <c r="E362" s="4" t="inlineStr">
         <is>
           <t>2631LZ27</t>
@@ -27494,9 +27770,7 @@
           <t>P</t>
         </is>
       </c>
-      <c r="D363" s="3" t="n">
-        <v>46264</v>
-      </c>
+      <c r="D363" s="3" t="n"/>
       <c r="E363" s="4" t="inlineStr">
         <is>
           <t>2631LY57</t>
@@ -27567,9 +27841,7 @@
           <t>P</t>
         </is>
       </c>
-      <c r="D364" s="3" t="n">
-        <v>46264</v>
-      </c>
+      <c r="D364" s="3" t="n"/>
       <c r="E364" s="4" t="inlineStr">
         <is>
           <t>2631LZ57</t>
@@ -27640,9 +27912,7 @@
           <t>P</t>
         </is>
       </c>
-      <c r="D365" s="3" t="n">
-        <v>46264</v>
-      </c>
+      <c r="D365" s="3" t="n"/>
       <c r="E365" s="4" t="inlineStr">
         <is>
           <t>2631HW17</t>
@@ -27713,9 +27983,7 @@
           <t>P</t>
         </is>
       </c>
-      <c r="D366" s="3" t="n">
-        <v>46264</v>
-      </c>
+      <c r="D366" s="3" t="n"/>
       <c r="E366" s="4" t="inlineStr">
         <is>
           <t>2631PK47</t>
@@ -27859,7 +28127,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D368" s="3" t="n"/>
+      <c r="D368" s="3" t="n">
+        <v>46257</v>
+      </c>
       <c r="E368" t="inlineStr">
         <is>
           <t>2629FX10</t>
@@ -27931,7 +28201,7 @@
         </is>
       </c>
       <c r="D369" s="3" t="n">
-        <v>46274</v>
+        <v>46257</v>
       </c>
       <c r="E369" t="inlineStr">
         <is>
@@ -28004,7 +28274,7 @@
         </is>
       </c>
       <c r="D370" s="3" t="n">
-        <v>46274</v>
+        <v>46279</v>
       </c>
       <c r="E370" t="inlineStr">
         <is>
@@ -28077,7 +28347,7 @@
         </is>
       </c>
       <c r="D371" s="3" t="n">
-        <v>46274</v>
+        <v>46279</v>
       </c>
       <c r="E371" t="inlineStr">
         <is>
@@ -28150,7 +28420,7 @@
         </is>
       </c>
       <c r="D372" s="3" t="n">
-        <v>46282</v>
+        <v>46279</v>
       </c>
       <c r="E372" t="inlineStr">
         <is>
@@ -28222,9 +28492,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D373" s="3" t="n">
-        <v>46282</v>
-      </c>
+      <c r="D373" s="3" t="n"/>
       <c r="E373" t="inlineStr">
         <is>
           <t>2631GD40</t>
@@ -28295,9 +28563,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D374" s="3" t="n">
-        <v>46282</v>
-      </c>
+      <c r="D374" s="3" t="n"/>
       <c r="E374" t="inlineStr">
         <is>
           <t>2631GD30</t>
@@ -28368,9 +28634,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="D375" s="3" t="n">
-        <v>46282</v>
-      </c>
+      <c r="D375" s="3" t="n"/>
       <c r="E375" t="inlineStr">
         <is>
           <t>2631GD50</t>
@@ -28515,7 +28779,7 @@
         </is>
       </c>
       <c r="D377" s="3" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -28588,7 +28852,7 @@
         </is>
       </c>
       <c r="D378" s="3" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="E378" t="inlineStr">
         <is>
@@ -28661,7 +28925,7 @@
         </is>
       </c>
       <c r="D379" s="3" t="n">
-        <v>46273</v>
+        <v>46268</v>
       </c>
       <c r="E379" t="inlineStr">
         <is>
@@ -28734,7 +28998,7 @@
         </is>
       </c>
       <c r="D380" s="3" t="n">
-        <v>46258</v>
+        <v>46268</v>
       </c>
       <c r="E380" t="inlineStr">
         <is>
@@ -29025,9 +29289,7 @@
           <t>P</t>
         </is>
       </c>
-      <c r="D384" s="3" t="n">
-        <v>46253</v>
-      </c>
+      <c r="D384" s="3" t="n"/>
       <c r="E384" s="4" t="inlineStr">
         <is>
           <t>2631DG67</t>

</xml_diff>

<commit_message>
Name the still-unmet date on the last lot when nothing is fully covered
If a part's very last available anode lot still leaves every date
("不够") uncovered, that last row now shows "<date> 还不够" - the
earliest date whose full-day demand remains unmet even after adding
every available lot - instead of a bare "不够". Earlier "不够" rows for
the same part are unchanged.

Verified against T598X156M075ATE075 in this run: rows 141-145 stay
"不够", and the last row (146, 2630FY30) now reads "2026-08-24 还不够".
</commit_message>
<xml_diff>
--- a/shortage_with_anode_report.xlsx
+++ b/shortage_with_anode_report.xlsx
@@ -4229,7 +4229,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-28 还不够</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -12289,7 +12289,7 @@
       </c>
       <c r="D146" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24 还不够</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -15211,7 +15211,7 @@
       </c>
       <c r="D186" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-28 还不够</t>
         </is>
       </c>
       <c r="E186" s="4" t="inlineStr">
@@ -22186,7 +22186,7 @@
       </c>
       <c r="D279" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24 还不够</t>
         </is>
       </c>
       <c r="E279" s="4" t="inlineStr">
@@ -25507,7 +25507,7 @@
       </c>
       <c r="D324" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-21 还不够</t>
         </is>
       </c>
       <c r="E324" s="4" t="inlineStr">
@@ -40412,7 +40412,7 @@
       </c>
       <c r="D525" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-09-03 还不够</t>
         </is>
       </c>
       <c r="E525" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Show the unmet date on every insufficient row, not just the last one
Replaces the plain "不够" text with "<date>不够" (the earliest date
whose full-day demand still isn't covered) on every row where the
running supply doesn't reach it yet, instead of reserving that detail
for the last available lot only.

Verified against T598X156M075ATE075: all 6 rows (141-146) now read
"2026-08-24不够" instead of a bare "不够".
</commit_message>
<xml_diff>
--- a/shortage_with_anode_report.xlsx
+++ b/shortage_with_anode_report.xlsx
@@ -3643,7 +3643,7 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-23不够</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -4229,7 +4229,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>2026-08-28 还不够</t>
+          <t>2026-08-28不够</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-09-07不够</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -4379,7 +4379,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-09-07不够</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -4454,7 +4454,7 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-09-07不够</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -4529,7 +4529,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-09-07不够</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -4604,7 +4604,7 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-09-07不够</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -4679,7 +4679,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-09-07不够</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -4754,7 +4754,7 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-09-07不够</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -4829,7 +4829,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-09-07不够</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -6729,7 +6729,7 @@
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-31不够</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
@@ -11914,7 +11914,7 @@
       </c>
       <c r="D141" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -11989,7 +11989,7 @@
       </c>
       <c r="D142" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -12064,7 +12064,7 @@
       </c>
       <c r="D143" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -12139,7 +12139,7 @@
       </c>
       <c r="D144" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -12214,7 +12214,7 @@
       </c>
       <c r="D145" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -12289,7 +12289,7 @@
       </c>
       <c r="D146" s="3" t="inlineStr">
         <is>
-          <t>2026-08-24 还不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -15211,7 +15211,7 @@
       </c>
       <c r="D186" s="3" t="inlineStr">
         <is>
-          <t>2026-08-28 还不够</t>
+          <t>2026-08-28不够</t>
         </is>
       </c>
       <c r="E186" s="4" t="inlineStr">
@@ -15286,7 +15286,7 @@
       </c>
       <c r="D187" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E187" s="4" t="inlineStr">
@@ -15361,7 +15361,7 @@
       </c>
       <c r="D188" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E188" s="4" t="inlineStr">
@@ -15436,7 +15436,7 @@
       </c>
       <c r="D189" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E189" s="4" t="inlineStr">
@@ -15511,7 +15511,7 @@
       </c>
       <c r="D190" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E190" s="4" t="inlineStr">
@@ -15586,7 +15586,7 @@
       </c>
       <c r="D191" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E191" s="4" t="inlineStr">
@@ -15661,7 +15661,7 @@
       </c>
       <c r="D192" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E192" s="4" t="inlineStr">
@@ -15736,7 +15736,7 @@
       </c>
       <c r="D193" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E193" s="4" t="inlineStr">
@@ -15811,7 +15811,7 @@
       </c>
       <c r="D194" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E194" s="4" t="inlineStr">
@@ -15886,7 +15886,7 @@
       </c>
       <c r="D195" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E195" s="4" t="inlineStr">
@@ -15961,7 +15961,7 @@
       </c>
       <c r="D196" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E196" s="4" t="inlineStr">
@@ -16036,7 +16036,7 @@
       </c>
       <c r="D197" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E197" s="4" t="inlineStr">
@@ -16111,7 +16111,7 @@
       </c>
       <c r="D198" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E198" s="4" t="inlineStr">
@@ -16186,7 +16186,7 @@
       </c>
       <c r="D199" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E199" s="4" t="inlineStr">
@@ -16261,7 +16261,7 @@
       </c>
       <c r="D200" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E200" s="4" t="inlineStr">
@@ -16336,7 +16336,7 @@
       </c>
       <c r="D201" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E201" s="4" t="inlineStr">
@@ -16411,7 +16411,7 @@
       </c>
       <c r="D202" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E202" s="4" t="inlineStr">
@@ -16486,7 +16486,7 @@
       </c>
       <c r="D203" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E203" s="4" t="inlineStr">
@@ -16561,7 +16561,7 @@
       </c>
       <c r="D204" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E204" s="4" t="inlineStr">
@@ -16636,7 +16636,7 @@
       </c>
       <c r="D205" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E205" s="4" t="inlineStr">
@@ -16711,7 +16711,7 @@
       </c>
       <c r="D206" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E206" s="4" t="inlineStr">
@@ -16786,7 +16786,7 @@
       </c>
       <c r="D207" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E207" s="4" t="inlineStr">
@@ -16861,7 +16861,7 @@
       </c>
       <c r="D208" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E208" s="4" t="inlineStr">
@@ -16936,7 +16936,7 @@
       </c>
       <c r="D209" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E209" s="4" t="inlineStr">
@@ -17011,7 +17011,7 @@
       </c>
       <c r="D210" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E210" s="4" t="inlineStr">
@@ -17086,7 +17086,7 @@
       </c>
       <c r="D211" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E211" s="4" t="inlineStr">
@@ -17161,7 +17161,7 @@
       </c>
       <c r="D212" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E212" s="4" t="inlineStr">
@@ -17236,7 +17236,7 @@
       </c>
       <c r="D213" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E213" s="4" t="inlineStr">
@@ -17311,7 +17311,7 @@
       </c>
       <c r="D214" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E214" s="4" t="inlineStr">
@@ -17386,7 +17386,7 @@
       </c>
       <c r="D215" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E215" s="4" t="inlineStr">
@@ -17461,7 +17461,7 @@
       </c>
       <c r="D216" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E216" s="4" t="inlineStr">
@@ -17536,7 +17536,7 @@
       </c>
       <c r="D217" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E217" s="4" t="inlineStr">
@@ -17611,7 +17611,7 @@
       </c>
       <c r="D218" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E218" s="4" t="inlineStr">
@@ -17686,7 +17686,7 @@
       </c>
       <c r="D219" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E219" s="4" t="inlineStr">
@@ -17761,7 +17761,7 @@
       </c>
       <c r="D220" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E220" s="4" t="inlineStr">
@@ -17836,7 +17836,7 @@
       </c>
       <c r="D221" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E221" s="4" t="inlineStr">
@@ -17911,7 +17911,7 @@
       </c>
       <c r="D222" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E222" s="4" t="inlineStr">
@@ -17986,7 +17986,7 @@
       </c>
       <c r="D223" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E223" s="4" t="inlineStr">
@@ -18061,7 +18061,7 @@
       </c>
       <c r="D224" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E224" s="4" t="inlineStr">
@@ -18136,7 +18136,7 @@
       </c>
       <c r="D225" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E225" s="4" t="inlineStr">
@@ -18211,7 +18211,7 @@
       </c>
       <c r="D226" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E226" s="4" t="inlineStr">
@@ -18286,7 +18286,7 @@
       </c>
       <c r="D227" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E227" s="4" t="inlineStr">
@@ -18361,7 +18361,7 @@
       </c>
       <c r="D228" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E228" s="4" t="inlineStr">
@@ -18436,7 +18436,7 @@
       </c>
       <c r="D229" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E229" s="4" t="inlineStr">
@@ -18511,7 +18511,7 @@
       </c>
       <c r="D230" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E230" s="4" t="inlineStr">
@@ -18586,7 +18586,7 @@
       </c>
       <c r="D231" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E231" s="4" t="inlineStr">
@@ -18661,7 +18661,7 @@
       </c>
       <c r="D232" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E232" s="4" t="inlineStr">
@@ -18736,7 +18736,7 @@
       </c>
       <c r="D233" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E233" s="4" t="inlineStr">
@@ -18811,7 +18811,7 @@
       </c>
       <c r="D234" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E234" s="4" t="inlineStr">
@@ -18886,7 +18886,7 @@
       </c>
       <c r="D235" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E235" s="4" t="inlineStr">
@@ -18961,7 +18961,7 @@
       </c>
       <c r="D236" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E236" s="4" t="inlineStr">
@@ -19036,7 +19036,7 @@
       </c>
       <c r="D237" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E237" s="4" t="inlineStr">
@@ -19111,7 +19111,7 @@
       </c>
       <c r="D238" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E238" s="4" t="inlineStr">
@@ -19186,7 +19186,7 @@
       </c>
       <c r="D239" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E239" s="4" t="inlineStr">
@@ -19261,7 +19261,7 @@
       </c>
       <c r="D240" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E240" s="4" t="inlineStr">
@@ -19336,7 +19336,7 @@
       </c>
       <c r="D241" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E241" s="4" t="inlineStr">
@@ -19411,7 +19411,7 @@
       </c>
       <c r="D242" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E242" s="4" t="inlineStr">
@@ -19486,7 +19486,7 @@
       </c>
       <c r="D243" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E243" s="4" t="inlineStr">
@@ -19561,7 +19561,7 @@
       </c>
       <c r="D244" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E244" s="4" t="inlineStr">
@@ -19636,7 +19636,7 @@
       </c>
       <c r="D245" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E245" s="4" t="inlineStr">
@@ -19711,7 +19711,7 @@
       </c>
       <c r="D246" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E246" s="4" t="inlineStr">
@@ -19786,7 +19786,7 @@
       </c>
       <c r="D247" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E247" s="4" t="inlineStr">
@@ -19861,7 +19861,7 @@
       </c>
       <c r="D248" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E248" s="4" t="inlineStr">
@@ -19936,7 +19936,7 @@
       </c>
       <c r="D249" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E249" s="4" t="inlineStr">
@@ -20011,7 +20011,7 @@
       </c>
       <c r="D250" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E250" s="4" t="inlineStr">
@@ -20086,7 +20086,7 @@
       </c>
       <c r="D251" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E251" s="4" t="inlineStr">
@@ -20161,7 +20161,7 @@
       </c>
       <c r="D252" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E252" s="4" t="inlineStr">
@@ -20236,7 +20236,7 @@
       </c>
       <c r="D253" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E253" s="4" t="inlineStr">
@@ -20311,7 +20311,7 @@
       </c>
       <c r="D254" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E254" s="4" t="inlineStr">
@@ -20386,7 +20386,7 @@
       </c>
       <c r="D255" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E255" s="4" t="inlineStr">
@@ -20461,7 +20461,7 @@
       </c>
       <c r="D256" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E256" s="4" t="inlineStr">
@@ -20536,7 +20536,7 @@
       </c>
       <c r="D257" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E257" s="4" t="inlineStr">
@@ -20611,7 +20611,7 @@
       </c>
       <c r="D258" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E258" s="4" t="inlineStr">
@@ -20686,7 +20686,7 @@
       </c>
       <c r="D259" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E259" s="4" t="inlineStr">
@@ -20761,7 +20761,7 @@
       </c>
       <c r="D260" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E260" s="4" t="inlineStr">
@@ -20836,7 +20836,7 @@
       </c>
       <c r="D261" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E261" s="4" t="inlineStr">
@@ -20911,7 +20911,7 @@
       </c>
       <c r="D262" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E262" s="4" t="inlineStr">
@@ -20986,7 +20986,7 @@
       </c>
       <c r="D263" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E263" s="4" t="inlineStr">
@@ -21061,7 +21061,7 @@
       </c>
       <c r="D264" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E264" s="4" t="inlineStr">
@@ -21136,7 +21136,7 @@
       </c>
       <c r="D265" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E265" s="4" t="inlineStr">
@@ -21211,7 +21211,7 @@
       </c>
       <c r="D266" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E266" s="4" t="inlineStr">
@@ -21286,7 +21286,7 @@
       </c>
       <c r="D267" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E267" s="4" t="inlineStr">
@@ -21361,7 +21361,7 @@
       </c>
       <c r="D268" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E268" s="4" t="inlineStr">
@@ -21436,7 +21436,7 @@
       </c>
       <c r="D269" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E269" s="4" t="inlineStr">
@@ -21511,7 +21511,7 @@
       </c>
       <c r="D270" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E270" s="4" t="inlineStr">
@@ -21586,7 +21586,7 @@
       </c>
       <c r="D271" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E271" s="4" t="inlineStr">
@@ -21661,7 +21661,7 @@
       </c>
       <c r="D272" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E272" s="4" t="inlineStr">
@@ -21736,7 +21736,7 @@
       </c>
       <c r="D273" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E273" s="4" t="inlineStr">
@@ -21811,7 +21811,7 @@
       </c>
       <c r="D274" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E274" s="4" t="inlineStr">
@@ -21886,7 +21886,7 @@
       </c>
       <c r="D275" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E275" s="4" t="inlineStr">
@@ -21961,7 +21961,7 @@
       </c>
       <c r="D276" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E276" s="4" t="inlineStr">
@@ -22036,7 +22036,7 @@
       </c>
       <c r="D277" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E277" s="4" t="inlineStr">
@@ -22111,7 +22111,7 @@
       </c>
       <c r="D278" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E278" s="4" t="inlineStr">
@@ -22186,7 +22186,7 @@
       </c>
       <c r="D279" s="3" t="inlineStr">
         <is>
-          <t>2026-08-24 还不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E279" s="4" t="inlineStr">
@@ -24232,7 +24232,7 @@
       </c>
       <c r="D307" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-21不够</t>
         </is>
       </c>
       <c r="E307" s="4" t="inlineStr">
@@ -24307,7 +24307,7 @@
       </c>
       <c r="D308" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-21不够</t>
         </is>
       </c>
       <c r="E308" s="4" t="inlineStr">
@@ -24382,7 +24382,7 @@
       </c>
       <c r="D309" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-21不够</t>
         </is>
       </c>
       <c r="E309" s="4" t="inlineStr">
@@ -24457,7 +24457,7 @@
       </c>
       <c r="D310" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-21不够</t>
         </is>
       </c>
       <c r="E310" s="4" t="inlineStr">
@@ -24532,7 +24532,7 @@
       </c>
       <c r="D311" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-21不够</t>
         </is>
       </c>
       <c r="E311" s="4" t="inlineStr">
@@ -24607,7 +24607,7 @@
       </c>
       <c r="D312" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-21不够</t>
         </is>
       </c>
       <c r="E312" s="4" t="inlineStr">
@@ -24682,7 +24682,7 @@
       </c>
       <c r="D313" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-21不够</t>
         </is>
       </c>
       <c r="E313" s="4" t="inlineStr">
@@ -24757,7 +24757,7 @@
       </c>
       <c r="D314" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-21不够</t>
         </is>
       </c>
       <c r="E314" s="4" t="inlineStr">
@@ -24832,7 +24832,7 @@
       </c>
       <c r="D315" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-21不够</t>
         </is>
       </c>
       <c r="E315" s="4" t="inlineStr">
@@ -24907,7 +24907,7 @@
       </c>
       <c r="D316" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-21不够</t>
         </is>
       </c>
       <c r="E316" s="4" t="inlineStr">
@@ -24982,7 +24982,7 @@
       </c>
       <c r="D317" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-21不够</t>
         </is>
       </c>
       <c r="E317" s="4" t="inlineStr">
@@ -25057,7 +25057,7 @@
       </c>
       <c r="D318" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-21不够</t>
         </is>
       </c>
       <c r="E318" s="4" t="inlineStr">
@@ -25132,7 +25132,7 @@
       </c>
       <c r="D319" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-21不够</t>
         </is>
       </c>
       <c r="E319" s="4" t="inlineStr">
@@ -25207,7 +25207,7 @@
       </c>
       <c r="D320" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-21不够</t>
         </is>
       </c>
       <c r="E320" s="4" t="inlineStr">
@@ -25282,7 +25282,7 @@
       </c>
       <c r="D321" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-21不够</t>
         </is>
       </c>
       <c r="E321" s="4" t="inlineStr">
@@ -25357,7 +25357,7 @@
       </c>
       <c r="D322" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-21不够</t>
         </is>
       </c>
       <c r="E322" s="4" t="inlineStr">
@@ -25432,7 +25432,7 @@
       </c>
       <c r="D323" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-21不够</t>
         </is>
       </c>
       <c r="E323" s="4" t="inlineStr">
@@ -25507,7 +25507,7 @@
       </c>
       <c r="D324" s="3" t="inlineStr">
         <is>
-          <t>2026-08-21 还不够</t>
+          <t>2026-08-21不够</t>
         </is>
       </c>
       <c r="E324" s="4" t="inlineStr">
@@ -26020,7 +26020,7 @@
       </c>
       <c r="D331" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E331" s="4" t="inlineStr">
@@ -26095,7 +26095,7 @@
       </c>
       <c r="D332" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E332" s="4" t="inlineStr">
@@ -26170,7 +26170,7 @@
       </c>
       <c r="D333" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E333" s="4" t="inlineStr">
@@ -26245,7 +26245,7 @@
       </c>
       <c r="D334" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E334" s="4" t="inlineStr">
@@ -26320,7 +26320,7 @@
       </c>
       <c r="D335" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E335" s="4" t="inlineStr">
@@ -26395,7 +26395,7 @@
       </c>
       <c r="D336" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E336" s="4" t="inlineStr">
@@ -26470,7 +26470,7 @@
       </c>
       <c r="D337" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E337" s="4" t="inlineStr">
@@ -26545,7 +26545,7 @@
       </c>
       <c r="D338" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E338" s="4" t="inlineStr">
@@ -26620,7 +26620,7 @@
       </c>
       <c r="D339" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E339" s="4" t="inlineStr">
@@ -26695,7 +26695,7 @@
       </c>
       <c r="D340" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E340" s="4" t="inlineStr">
@@ -26770,7 +26770,7 @@
       </c>
       <c r="D341" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E341" s="4" t="inlineStr">
@@ -26845,7 +26845,7 @@
       </c>
       <c r="D342" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E342" s="4" t="inlineStr">
@@ -26920,7 +26920,7 @@
       </c>
       <c r="D343" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E343" s="4" t="inlineStr">
@@ -26995,7 +26995,7 @@
       </c>
       <c r="D344" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E344" s="4" t="inlineStr">
@@ -27070,7 +27070,7 @@
       </c>
       <c r="D345" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E345" s="4" t="inlineStr">
@@ -27145,7 +27145,7 @@
       </c>
       <c r="D346" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E346" s="4" t="inlineStr">
@@ -27220,7 +27220,7 @@
       </c>
       <c r="D347" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E347" s="4" t="inlineStr">
@@ -27295,7 +27295,7 @@
       </c>
       <c r="D348" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E348" s="4" t="inlineStr">
@@ -27370,7 +27370,7 @@
       </c>
       <c r="D349" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E349" s="4" t="inlineStr">
@@ -27445,7 +27445,7 @@
       </c>
       <c r="D350" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E350" s="4" t="inlineStr">
@@ -27520,7 +27520,7 @@
       </c>
       <c r="D351" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E351" s="4" t="inlineStr">
@@ -27595,7 +27595,7 @@
       </c>
       <c r="D352" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E352" s="4" t="inlineStr">
@@ -27670,7 +27670,7 @@
       </c>
       <c r="D353" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E353" s="4" t="inlineStr">
@@ -27745,7 +27745,7 @@
       </c>
       <c r="D354" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E354" s="4" t="inlineStr">
@@ -27820,7 +27820,7 @@
       </c>
       <c r="D355" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E355" s="4" t="inlineStr">
@@ -27895,7 +27895,7 @@
       </c>
       <c r="D356" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E356" s="4" t="inlineStr">
@@ -27970,7 +27970,7 @@
       </c>
       <c r="D357" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E357" s="4" t="inlineStr">
@@ -28045,7 +28045,7 @@
       </c>
       <c r="D358" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E358" s="4" t="inlineStr">
@@ -28120,7 +28120,7 @@
       </c>
       <c r="D359" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E359" s="4" t="inlineStr">
@@ -28195,7 +28195,7 @@
       </c>
       <c r="D360" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E360" s="4" t="inlineStr">
@@ -28270,7 +28270,7 @@
       </c>
       <c r="D361" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E361" s="4" t="inlineStr">
@@ -28345,7 +28345,7 @@
       </c>
       <c r="D362" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E362" s="4" t="inlineStr">
@@ -28420,7 +28420,7 @@
       </c>
       <c r="D363" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E363" s="4" t="inlineStr">
@@ -28495,7 +28495,7 @@
       </c>
       <c r="D364" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E364" s="4" t="inlineStr">
@@ -28570,7 +28570,7 @@
       </c>
       <c r="D365" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E365" s="4" t="inlineStr">
@@ -28645,7 +28645,7 @@
       </c>
       <c r="D366" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E366" s="4" t="inlineStr">
@@ -28720,7 +28720,7 @@
       </c>
       <c r="D367" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E367" s="4" t="inlineStr">
@@ -28795,7 +28795,7 @@
       </c>
       <c r="D368" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E368" s="4" t="inlineStr">
@@ -28870,7 +28870,7 @@
       </c>
       <c r="D369" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E369" s="4" t="inlineStr">
@@ -28945,7 +28945,7 @@
       </c>
       <c r="D370" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E370" s="4" t="inlineStr">
@@ -29020,7 +29020,7 @@
       </c>
       <c r="D371" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E371" s="4" t="inlineStr">
@@ -29095,7 +29095,7 @@
       </c>
       <c r="D372" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E372" s="4" t="inlineStr">
@@ -29170,7 +29170,7 @@
       </c>
       <c r="D373" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E373" s="4" t="inlineStr">
@@ -29245,7 +29245,7 @@
       </c>
       <c r="D374" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E374" s="4" t="inlineStr">
@@ -29320,7 +29320,7 @@
       </c>
       <c r="D375" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E375" s="4" t="inlineStr">
@@ -29395,7 +29395,7 @@
       </c>
       <c r="D376" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E376" s="4" t="inlineStr">
@@ -29470,7 +29470,7 @@
       </c>
       <c r="D377" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E377" s="4" t="inlineStr">
@@ -29545,7 +29545,7 @@
       </c>
       <c r="D378" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E378" s="4" t="inlineStr">
@@ -29620,7 +29620,7 @@
       </c>
       <c r="D379" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E379" s="4" t="inlineStr">
@@ -29695,7 +29695,7 @@
       </c>
       <c r="D380" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E380" s="4" t="inlineStr">
@@ -29770,7 +29770,7 @@
       </c>
       <c r="D381" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E381" s="4" t="inlineStr">
@@ -29845,7 +29845,7 @@
       </c>
       <c r="D382" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E382" s="4" t="inlineStr">
@@ -29920,7 +29920,7 @@
       </c>
       <c r="D383" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E383" s="4" t="inlineStr">
@@ -29995,7 +29995,7 @@
       </c>
       <c r="D384" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E384" s="4" t="inlineStr">
@@ -30070,7 +30070,7 @@
       </c>
       <c r="D385" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E385" s="4" t="inlineStr">
@@ -30145,7 +30145,7 @@
       </c>
       <c r="D386" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E386" s="4" t="inlineStr">
@@ -30220,7 +30220,7 @@
       </c>
       <c r="D387" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E387" s="4" t="inlineStr">
@@ -30295,7 +30295,7 @@
       </c>
       <c r="D388" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E388" s="4" t="inlineStr">
@@ -30370,7 +30370,7 @@
       </c>
       <c r="D389" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E389" s="4" t="inlineStr">
@@ -30445,7 +30445,7 @@
       </c>
       <c r="D390" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E390" s="4" t="inlineStr">
@@ -30520,7 +30520,7 @@
       </c>
       <c r="D391" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E391" s="4" t="inlineStr">
@@ -30595,7 +30595,7 @@
       </c>
       <c r="D392" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E392" s="4" t="inlineStr">
@@ -30670,7 +30670,7 @@
       </c>
       <c r="D393" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E393" s="4" t="inlineStr">
@@ -30745,7 +30745,7 @@
       </c>
       <c r="D394" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E394" s="4" t="inlineStr">
@@ -30820,7 +30820,7 @@
       </c>
       <c r="D395" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E395" s="4" t="inlineStr">
@@ -30895,7 +30895,7 @@
       </c>
       <c r="D396" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E396" s="4" t="inlineStr">
@@ -30970,7 +30970,7 @@
       </c>
       <c r="D397" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E397" s="4" t="inlineStr">
@@ -31045,7 +31045,7 @@
       </c>
       <c r="D398" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E398" s="4" t="inlineStr">
@@ -31120,7 +31120,7 @@
       </c>
       <c r="D399" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E399" s="4" t="inlineStr">
@@ -31195,7 +31195,7 @@
       </c>
       <c r="D400" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E400" s="4" t="inlineStr">
@@ -31270,7 +31270,7 @@
       </c>
       <c r="D401" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E401" s="4" t="inlineStr">
@@ -31345,7 +31345,7 @@
       </c>
       <c r="D402" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E402" s="4" t="inlineStr">
@@ -31420,7 +31420,7 @@
       </c>
       <c r="D403" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E403" s="4" t="inlineStr">
@@ -31495,7 +31495,7 @@
       </c>
       <c r="D404" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E404" s="4" t="inlineStr">
@@ -31570,7 +31570,7 @@
       </c>
       <c r="D405" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E405" s="4" t="inlineStr">
@@ -31645,7 +31645,7 @@
       </c>
       <c r="D406" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E406" s="4" t="inlineStr">
@@ -31720,7 +31720,7 @@
       </c>
       <c r="D407" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E407" s="4" t="inlineStr">
@@ -31795,7 +31795,7 @@
       </c>
       <c r="D408" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E408" s="4" t="inlineStr">
@@ -31870,7 +31870,7 @@
       </c>
       <c r="D409" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E409" s="4" t="inlineStr">
@@ -31945,7 +31945,7 @@
       </c>
       <c r="D410" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E410" s="4" t="inlineStr">
@@ -32020,7 +32020,7 @@
       </c>
       <c r="D411" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E411" s="4" t="inlineStr">
@@ -32095,7 +32095,7 @@
       </c>
       <c r="D412" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E412" s="4" t="inlineStr">
@@ -32170,7 +32170,7 @@
       </c>
       <c r="D413" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E413" s="4" t="inlineStr">
@@ -32245,7 +32245,7 @@
       </c>
       <c r="D414" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E414" s="4" t="inlineStr">
@@ -32320,7 +32320,7 @@
       </c>
       <c r="D415" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E415" s="4" t="inlineStr">
@@ -32395,7 +32395,7 @@
       </c>
       <c r="D416" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E416" s="4" t="inlineStr">
@@ -32470,7 +32470,7 @@
       </c>
       <c r="D417" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E417" s="4" t="inlineStr">
@@ -32545,7 +32545,7 @@
       </c>
       <c r="D418" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E418" s="4" t="inlineStr">
@@ -32620,7 +32620,7 @@
       </c>
       <c r="D419" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E419" s="4" t="inlineStr">
@@ -32695,7 +32695,7 @@
       </c>
       <c r="D420" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E420" s="4" t="inlineStr">
@@ -32989,7 +32989,7 @@
       </c>
       <c r="D424" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E424" s="4" t="inlineStr">
@@ -33064,7 +33064,7 @@
       </c>
       <c r="D425" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E425" s="4" t="inlineStr">
@@ -33139,7 +33139,7 @@
       </c>
       <c r="D426" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E426" s="4" t="inlineStr">
@@ -33214,7 +33214,7 @@
       </c>
       <c r="D427" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E427" s="4" t="inlineStr">
@@ -33289,7 +33289,7 @@
       </c>
       <c r="D428" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E428" s="4" t="inlineStr">
@@ -33364,7 +33364,7 @@
       </c>
       <c r="D429" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E429" s="4" t="inlineStr">
@@ -33439,7 +33439,7 @@
       </c>
       <c r="D430" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E430" s="4" t="inlineStr">
@@ -33514,7 +33514,7 @@
       </c>
       <c r="D431" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E431" s="4" t="inlineStr">
@@ -33589,7 +33589,7 @@
       </c>
       <c r="D432" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E432" s="4" t="inlineStr">
@@ -33664,7 +33664,7 @@
       </c>
       <c r="D433" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E433" s="4" t="inlineStr">
@@ -33739,7 +33739,7 @@
       </c>
       <c r="D434" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E434" s="4" t="inlineStr">
@@ -33814,7 +33814,7 @@
       </c>
       <c r="D435" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E435" s="4" t="inlineStr">
@@ -33889,7 +33889,7 @@
       </c>
       <c r="D436" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E436" s="4" t="inlineStr">
@@ -33964,7 +33964,7 @@
       </c>
       <c r="D437" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E437" s="4" t="inlineStr">
@@ -34039,7 +34039,7 @@
       </c>
       <c r="D438" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E438" s="4" t="inlineStr">
@@ -34114,7 +34114,7 @@
       </c>
       <c r="D439" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E439" s="4" t="inlineStr">
@@ -34189,7 +34189,7 @@
       </c>
       <c r="D440" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E440" s="4" t="inlineStr">
@@ -34264,7 +34264,7 @@
       </c>
       <c r="D441" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E441" s="4" t="inlineStr">
@@ -34339,7 +34339,7 @@
       </c>
       <c r="D442" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E442" s="4" t="inlineStr">
@@ -34414,7 +34414,7 @@
       </c>
       <c r="D443" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E443" s="4" t="inlineStr">
@@ -34489,7 +34489,7 @@
       </c>
       <c r="D444" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E444" s="4" t="inlineStr">
@@ -34564,7 +34564,7 @@
       </c>
       <c r="D445" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E445" s="4" t="inlineStr">
@@ -34639,7 +34639,7 @@
       </c>
       <c r="D446" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E446" s="4" t="inlineStr">
@@ -34714,7 +34714,7 @@
       </c>
       <c r="D447" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E447" s="4" t="inlineStr">
@@ -34789,7 +34789,7 @@
       </c>
       <c r="D448" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-24不够</t>
         </is>
       </c>
       <c r="E448" s="4" t="inlineStr">
@@ -40412,7 +40412,7 @@
       </c>
       <c r="D525" s="3" t="inlineStr">
         <is>
-          <t>2026-09-03 还不够</t>
+          <t>2026-09-03不够</t>
         </is>
       </c>
       <c r="E525" s="4" t="inlineStr">
@@ -40925,7 +40925,7 @@
       </c>
       <c r="D532" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-22不够</t>
         </is>
       </c>
       <c r="E532" s="4" t="inlineStr">
@@ -41000,7 +41000,7 @@
       </c>
       <c r="D533" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-22不够</t>
         </is>
       </c>
       <c r="E533" s="4" t="inlineStr">
@@ -41075,7 +41075,7 @@
       </c>
       <c r="D534" s="3" t="inlineStr">
         <is>
-          <t>不够</t>
+          <t>2026-08-22不够</t>
         </is>
       </c>
       <c r="E534" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Add per-category AE (Kpcs/Cycles) threshold overrides
New repeatable --category-threshold "CATEGORY=VALUE" CLI option lets
specific Anode Categories (Loading sheet column A) use a different AE
threshold than the global --kpcs-threshold default. Each demand row's
own category is looked up against the override map; unlisted
categories keep using --kpcs-threshold. Recorded in the output's
Parameters sheet alongside the default.

Regenerated shortage_with_anode_report.xlsx with no overrides applied
(same 32 shortage parts as before), confirming the change is additive
and doesn't affect existing behavior when the option is unused.
</commit_message>
<xml_diff>
--- a/shortage_with_anode_report.xlsx
+++ b/shortage_with_anode_report.xlsx
@@ -43481,7 +43481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -43563,7 +43563,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>kpcs_threshold (AE column, strictly greater than)</t>
+          <t>kpcs_threshold (AE column, strictly greater than, default for unlisted categories)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -43575,10 +43575,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>category_thresholds (AE, strictly greater than, per Anode Category)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>(none)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>anode_cutoff_date (Intransit WAYBILL date, on or before cutoff)</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>

</xml_diff>